<commit_message>
Deployed 0552288 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/assets/fiche-personnage-hxh.xlsx
+++ b/assets/fiche-personnage-hxh.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0\%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +63,11 @@
       <i val="1"/>
       <color rgb="00555555"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF1D1D1D"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="10">
@@ -113,7 +118,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -212,11 +217,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -280,6 +286,19 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -646,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N140"/>
+  <dimension ref="A1:Q140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -671,19 +690,19 @@
           <t>FICHE DE PERSONNAGE — Hunter × Hunter (JDR)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="2" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="9" t="n"/>
+      <c r="D1" s="9" t="n"/>
+      <c r="E1" s="9" t="n"/>
+      <c r="F1" s="9" t="n"/>
+      <c r="G1" s="9" t="n"/>
+      <c r="H1" s="9" t="n"/>
+      <c r="I1" s="9" t="n"/>
+      <c r="J1" s="9" t="n"/>
+      <c r="K1" s="9" t="n"/>
+      <c r="L1" s="9" t="n"/>
+      <c r="M1" s="9" t="n"/>
+      <c r="N1" s="10" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -691,19 +710,19 @@
           <t>Légende : cellules BLANCHES = à remplir (saisie) ;  cellules BEIGES = calculées automatiquement (ne pas écrire dedans).</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
+      <c r="B2" s="9" t="n"/>
+      <c r="C2" s="9" t="n"/>
+      <c r="D2" s="9" t="n"/>
+      <c r="E2" s="9" t="n"/>
+      <c r="F2" s="9" t="n"/>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n"/>
+      <c r="I2" s="9" t="n"/>
+      <c r="J2" s="9" t="n"/>
+      <c r="K2" s="9" t="n"/>
+      <c r="L2" s="9" t="n"/>
+      <c r="M2" s="9" t="n"/>
+      <c r="N2" s="10" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -711,19 +730,19 @@
           <t>1 · Identité</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="n"/>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
-      <c r="M4" s="6" t="n"/>
-      <c r="N4" s="6" t="n"/>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="9" t="n"/>
+      <c r="J4" s="9" t="n"/>
+      <c r="K4" s="9" t="n"/>
+      <c r="L4" s="9" t="n"/>
+      <c r="M4" s="9" t="n"/>
+      <c r="N4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -873,19 +892,19 @@
           <t>1 bis · Plafonds de formation (Combattant)</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="n"/>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="6" t="n"/>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="6" t="n"/>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="9" t="n"/>
+      <c r="N12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
@@ -944,121 +963,145 @@
         <v>40</v>
       </c>
       <c r="C14" s="12">
-        <f>ROUNDDOWN(40*$B$7/100,0)</f>
+        <f>ROUNDDOWN(B14*$B$7/100,0)</f>
         <v/>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Furtif</t>
+          <t>Intellectuel</t>
         </is>
       </c>
       <c r="G14" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H14" s="12">
+        <f>ROUNDDOWN(G14*$B$7/100,0)</f>
+        <v/>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="L14" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="H14" s="12">
-        <f>ROUNDDOWN(20*$B$7/100,0)</f>
-        <v/>
-      </c>
-      <c r="K14" s="7" t="inlineStr">
-        <is>
-          <t>Intellectuel</t>
-        </is>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>10</v>
-      </c>
       <c r="M14" s="12">
-        <f>ROUNDDOWN(10*$B$7/100,0)</f>
+        <f>ROUNDDOWN(L14*$B$7/100,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Vital</t>
+          <t>Athlétique</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
         <v>30</v>
       </c>
       <c r="C15" s="12">
-        <f>ROUNDDOWN(30*$B$7/100,0)</f>
+        <f>ROUNDDOWN(B15*$B$7/100,0)</f>
         <v/>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Sauvage</t>
+          <t>Naturel</t>
         </is>
       </c>
       <c r="G15" s="15" t="n">
         <v>20</v>
       </c>
       <c r="H15" s="12">
-        <f>ROUNDDOWN(20*$B$7/100,0)</f>
+        <f>ROUNDDOWN(G15*$B$7/100,0)</f>
         <v/>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>Technique</t>
+          <t>Furtif</t>
         </is>
       </c>
       <c r="L15" s="15" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="M15" s="12">
-        <f>ROUNDDOWN(10*$B$7/100,0)</f>
+        <f>ROUNDDOWN(L15*$B$7/100,0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Athlétique</t>
+          <t>Vital</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
         <v>30</v>
       </c>
       <c r="C16" s="12">
-        <f>ROUNDDOWN(30*$B$7/100,0)</f>
+        <f>ROUNDDOWN(B16*$B$7/100,0)</f>
         <v/>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Social</t>
+          <t>Sensoriel</t>
         </is>
       </c>
       <c r="G16" s="15" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H16" s="12">
-        <f>ROUNDDOWN(10*$B$7/100,0)</f>
+        <f>ROUNDDOWN(G16*$B$7/100,0)</f>
         <v/>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Créatif</t>
+          <t>Artisanal</t>
         </is>
       </c>
       <c r="L16" s="15" t="n">
         <v>10</v>
       </c>
       <c r="M16" s="12">
-        <f>ROUNDDOWN(10*$B$7/100,0)</f>
+        <f>ROUNDDOWN(L16*$B$7/100,0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Sensoriel</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C17" s="12">
-        <f>ROUNDDOWN(20*$B$7/100,0)</f>
+        <f>ROUNDDOWN(B17*$B$7/100,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H17" s="12">
+        <f>ROUNDDOWN(G17*$B$7/100,0)</f>
+        <v/>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>Artistique</t>
+        </is>
+      </c>
+      <c r="L17" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="M17" s="12">
+        <f>ROUNDDOWN(L17*$B$7/100,0)</f>
         <v/>
       </c>
     </row>
@@ -1075,19 +1118,19 @@
           <t>2 · Caractéristiques  (saisie 0–30, ≤ plafond)</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
-      <c r="J20" s="6" t="n"/>
-      <c r="K20" s="6" t="n"/>
-      <c r="L20" s="6" t="n"/>
-      <c r="M20" s="6" t="n"/>
-      <c r="N20" s="6" t="n"/>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="9" t="n"/>
+      <c r="F20" s="9" t="n"/>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9" t="n"/>
+      <c r="I20" s="9" t="n"/>
+      <c r="J20" s="9" t="n"/>
+      <c r="K20" s="9" t="n"/>
+      <c r="L20" s="9" t="n"/>
+      <c r="M20" s="9" t="n"/>
+      <c r="N20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
@@ -1130,6 +1173,19 @@
           <t>Plafond</t>
         </is>
       </c>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>Point buy — création</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="n"/>
+      <c r="M21" s="9" t="n"/>
+      <c r="N21" s="10" t="n"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>(aux. coût point-buy par carac)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1164,6 +1220,32 @@
         <f>$G$6</f>
         <v/>
       </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="L22" s="12">
+        <f>VLOOKUP($B$6,Barèmes!$A$48:$D$51,2,TRUE)</f>
+        <v/>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>Plafond</t>
+        </is>
+      </c>
+      <c r="N22" s="12">
+        <f>VLOOKUP($B$6,Barèmes!$A$48:$D$51,3,TRUE)</f>
+        <v/>
+      </c>
+      <c r="P22">
+        <f>IF(B22&lt;=$L$22,B22-3,($L$22-3)+(B22-$L$22)*(B22-$L$22+3)/2)</f>
+        <v/>
+      </c>
+      <c r="Q22">
+        <f>IF(G22&lt;=$L$22,G22-3,($L$22-3)+(G22-$L$22)*(G22-$L$22+3)/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1198,6 +1280,32 @@
         <f>$G$6</f>
         <v/>
       </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="L23" s="12">
+        <f>VLOOKUP($B$6,Barèmes!$A$48:$D$51,4,TRUE)</f>
+        <v/>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>Coût</t>
+        </is>
+      </c>
+      <c r="N23" s="12">
+        <f>SUM(P22:P27)+SUM(Q22:Q27)</f>
+        <v/>
+      </c>
+      <c r="P23">
+        <f>IF(B23&lt;=$L$22,B23-3,($L$22-3)+(B23-$L$22)*(B23-$L$22+3)/2)</f>
+        <v/>
+      </c>
+      <c r="Q23">
+        <f>IF(G23&lt;=$L$22,G23-3,($L$22-3)+(G23-$L$22)*(G23-$L$22+3)/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1232,6 +1340,32 @@
         <f>$G$6</f>
         <v/>
       </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>Reste</t>
+        </is>
+      </c>
+      <c r="L24" s="12">
+        <f>L23-N23</f>
+        <v/>
+      </c>
+      <c r="M24" s="7" t="inlineStr">
+        <is>
+          <t>&gt; plafond ?</t>
+        </is>
+      </c>
+      <c r="N24" s="12">
+        <f>IF(MAX(B22:B27,G22:G27)&gt;N22,"oui","non")</f>
+        <v/>
+      </c>
+      <c r="P24">
+        <f>IF(B24&lt;=$L$22,B24-3,($L$22-3)+(B24-$L$22)*(B24-$L$22+3)/2)</f>
+        <v/>
+      </c>
+      <c r="Q24">
+        <f>IF(G24&lt;=$L$22,G24-3,($L$22-3)+(G24-$L$22)*(G24-$L$22+3)/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1266,6 +1400,14 @@
         <f>$G$6</f>
         <v/>
       </c>
+      <c r="P25">
+        <f>IF(B25&lt;=$L$22,B25-3,($L$22-3)+(B25-$L$22)*(B25-$L$22+3)/2)</f>
+        <v/>
+      </c>
+      <c r="Q25">
+        <f>IF(G25&lt;=$L$22,G25-3,($L$22-3)+(G25-$L$22)*(G25-$L$22+3)/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1300,6 +1442,14 @@
         <f>$G$6</f>
         <v/>
       </c>
+      <c r="P26">
+        <f>IF(B26&lt;=$L$22,B26-3,($L$22-3)+(B26-$L$22)*(B26-$L$22+3)/2)</f>
+        <v/>
+      </c>
+      <c r="Q26">
+        <f>IF(G26&lt;=$L$22,G26-3,($L$22-3)+(G26-$L$22)*(G26-$L$22+3)/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1334,6 +1484,14 @@
         <f>$G$6</f>
         <v/>
       </c>
+      <c r="P27">
+        <f>IF(B27&lt;=$L$22,B27-3,($L$22-3)+(B27-$L$22)*(B27-$L$22+3)/2)</f>
+        <v/>
+      </c>
+      <c r="Q27">
+        <f>IF(G27&lt;=$L$22,G27-3,($L$22-3)+(G27-$L$22)*(G27-$L$22+3)/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1357,19 +1515,19 @@
           <t>3 · Capacités physiques</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
-      <c r="J30" s="6" t="n"/>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
-      <c r="M30" s="6" t="n"/>
-      <c r="N30" s="6" t="n"/>
+      <c r="B30" s="9" t="n"/>
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n"/>
+      <c r="I30" s="9" t="n"/>
+      <c r="J30" s="9" t="n"/>
+      <c r="K30" s="9" t="n"/>
+      <c r="L30" s="9" t="n"/>
+      <c r="M30" s="9" t="n"/>
+      <c r="N30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1551,19 +1709,19 @@
           <t>4 · Combat</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="6" t="n"/>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="6" t="n"/>
-      <c r="J37" s="6" t="n"/>
-      <c r="K37" s="6" t="n"/>
-      <c r="L37" s="6" t="n"/>
-      <c r="M37" s="6" t="n"/>
-      <c r="N37" s="6" t="n"/>
+      <c r="B37" s="9" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="9" t="n"/>
+      <c r="L37" s="9" t="n"/>
+      <c r="M37" s="9" t="n"/>
+      <c r="N37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -1597,7 +1755,7 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>TA (armure)</t>
+          <t>Réduction de dégâts (armure)</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
@@ -1735,7 +1893,7 @@
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t>Dégâts infligés = (Dégâts de base − TA du type) × marge% ; la TA se retire avant le multiplicateur.</t>
+          <t>Dégâts infligés = (Dégâts de base − réduction de dégâts du type) × marge% ; la réduction se retire avant le multiplicateur.</t>
         </is>
       </c>
     </row>
@@ -1745,19 +1903,19 @@
           <t>5 · Aura &amp; Nen</t>
         </is>
       </c>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="6" t="n"/>
-      <c r="D48" s="6" t="n"/>
-      <c r="E48" s="6" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="6" t="n"/>
-      <c r="H48" s="6" t="n"/>
-      <c r="I48" s="6" t="n"/>
-      <c r="J48" s="6" t="n"/>
-      <c r="K48" s="6" t="n"/>
-      <c r="L48" s="6" t="n"/>
-      <c r="M48" s="6" t="n"/>
-      <c r="N48" s="6" t="n"/>
+      <c r="B48" s="9" t="n"/>
+      <c r="C48" s="9" t="n"/>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="9" t="n"/>
+      <c r="F48" s="9" t="n"/>
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n"/>
+      <c r="I48" s="9" t="n"/>
+      <c r="J48" s="9" t="n"/>
+      <c r="K48" s="9" t="n"/>
+      <c r="L48" s="9" t="n"/>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2134,19 +2292,19 @@
           <t>6 · Techniques du Nen</t>
         </is>
       </c>
-      <c r="B64" s="6" t="n"/>
-      <c r="C64" s="6" t="n"/>
-      <c r="D64" s="6" t="n"/>
-      <c r="E64" s="6" t="n"/>
-      <c r="F64" s="6" t="n"/>
-      <c r="G64" s="6" t="n"/>
-      <c r="H64" s="6" t="n"/>
-      <c r="I64" s="6" t="n"/>
-      <c r="J64" s="6" t="n"/>
-      <c r="K64" s="6" t="n"/>
-      <c r="L64" s="6" t="n"/>
-      <c r="M64" s="6" t="n"/>
-      <c r="N64" s="6" t="n"/>
+      <c r="B64" s="9" t="n"/>
+      <c r="C64" s="9" t="n"/>
+      <c r="D64" s="9" t="n"/>
+      <c r="E64" s="9" t="n"/>
+      <c r="F64" s="9" t="n"/>
+      <c r="G64" s="9" t="n"/>
+      <c r="H64" s="9" t="n"/>
+      <c r="I64" s="9" t="n"/>
+      <c r="J64" s="9" t="n"/>
+      <c r="K64" s="9" t="n"/>
+      <c r="L64" s="9" t="n"/>
+      <c r="M64" s="9" t="n"/>
+      <c r="N64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
@@ -2393,19 +2551,19 @@
           <t>7 · Compétences  (Bonus = Valeur + MOD de la carac liée)</t>
         </is>
       </c>
-      <c r="B76" s="6" t="n"/>
-      <c r="C76" s="6" t="n"/>
-      <c r="D76" s="6" t="n"/>
-      <c r="E76" s="6" t="n"/>
-      <c r="F76" s="6" t="n"/>
-      <c r="G76" s="6" t="n"/>
-      <c r="H76" s="6" t="n"/>
-      <c r="I76" s="6" t="n"/>
-      <c r="J76" s="6" t="n"/>
-      <c r="K76" s="6" t="n"/>
-      <c r="L76" s="6" t="n"/>
-      <c r="M76" s="6" t="n"/>
-      <c r="N76" s="6" t="n"/>
+      <c r="B76" s="9" t="n"/>
+      <c r="C76" s="9" t="n"/>
+      <c r="D76" s="9" t="n"/>
+      <c r="E76" s="9" t="n"/>
+      <c r="F76" s="9" t="n"/>
+      <c r="G76" s="9" t="n"/>
+      <c r="H76" s="9" t="n"/>
+      <c r="I76" s="9" t="n"/>
+      <c r="J76" s="9" t="n"/>
+      <c r="K76" s="9" t="n"/>
+      <c r="L76" s="9" t="n"/>
+      <c r="M76" s="9" t="n"/>
+      <c r="N76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="19" t="inlineStr">
@@ -2413,25 +2571,27 @@
           <t>Champ Martial</t>
         </is>
       </c>
-      <c r="B77" s="6" t="n"/>
-      <c r="C77" s="6" t="n"/>
-      <c r="D77" s="6" t="n"/>
+      <c r="B77" s="9" t="n"/>
+      <c r="C77" s="9" t="n"/>
+      <c r="D77" s="10" t="n"/>
+      <c r="E77" s="26" t="n"/>
       <c r="F77" s="19" t="inlineStr">
         <is>
           <t>Champ Social</t>
         </is>
       </c>
-      <c r="G77" s="6" t="n"/>
-      <c r="H77" s="6" t="n"/>
-      <c r="I77" s="6" t="n"/>
+      <c r="G77" s="9" t="n"/>
+      <c r="H77" s="9" t="n"/>
+      <c r="I77" s="10" t="n"/>
+      <c r="J77" s="26" t="n"/>
       <c r="K77" s="19" t="inlineStr">
         <is>
           <t>Champ Intellectuel</t>
         </is>
       </c>
-      <c r="L77" s="6" t="n"/>
-      <c r="M77" s="6" t="n"/>
-      <c r="N77" s="6" t="n"/>
+      <c r="L77" s="9" t="n"/>
+      <c r="M77" s="9" t="n"/>
+      <c r="N77" s="10" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
@@ -2454,6 +2614,7 @@
           <t>Bonus</t>
         </is>
       </c>
+      <c r="E78" s="26" t="n"/>
       <c r="F78" s="14" t="inlineStr">
         <is>
           <t>Compétence</t>
@@ -2474,6 +2635,7 @@
           <t>Bonus</t>
         </is>
       </c>
+      <c r="J78" s="26" t="n"/>
       <c r="K78" s="14" t="inlineStr">
         <is>
           <t>Compétence</t>
@@ -2513,6 +2675,7 @@
         <f>C79+C24+10</f>
         <v/>
       </c>
+      <c r="E79" s="26" t="n"/>
       <c r="F79" s="20" t="inlineStr">
         <is>
           <t>Persuasion</t>
@@ -2530,6 +2693,7 @@
         <f>H79+H27</f>
         <v/>
       </c>
+      <c r="J79" s="26" t="n"/>
       <c r="K79" s="20" t="inlineStr">
         <is>
           <t>Histoire</t>
@@ -2549,12 +2713,12 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="22" t="inlineStr">
+      <c r="A80" s="20" t="inlineStr">
         <is>
           <t>Armes de mêlée</t>
         </is>
       </c>
-      <c r="B80" s="23" t="inlineStr">
+      <c r="B80" s="21" t="inlineStr">
         <is>
           <t>DEX</t>
         </is>
@@ -2563,32 +2727,34 @@
         <v>0</v>
       </c>
       <c r="D80" s="12">
-        <f>C80+C23+IF(B9="Armes de mêlée",10,0)</f>
-        <v/>
-      </c>
-      <c r="F80" s="22" t="inlineStr">
+        <f>C80+C23+IF($B$9="Armes de mêlée",10,0)</f>
+        <v/>
+      </c>
+      <c r="E80" s="26" t="n"/>
+      <c r="F80" s="20" t="inlineStr">
         <is>
           <t>Rhétorique</t>
         </is>
       </c>
-      <c r="G80" s="23" t="inlineStr">
-        <is>
-          <t>LOG</t>
+      <c r="G80" s="21" t="inlineStr">
+        <is>
+          <t>CHA</t>
         </is>
       </c>
       <c r="H80" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I80" s="12">
-        <f>H80+H23</f>
-        <v/>
-      </c>
-      <c r="K80" s="22" t="inlineStr">
+        <f>H80+H27</f>
+        <v/>
+      </c>
+      <c r="J80" s="26" t="n"/>
+      <c r="K80" s="20" t="inlineStr">
         <is>
           <t>Archéologie</t>
         </is>
       </c>
-      <c r="L80" s="23" t="inlineStr">
+      <c r="L80" s="21" t="inlineStr">
         <is>
           <t>ÉRU</t>
         </is>
@@ -2616,9 +2782,10 @@
         <v>0</v>
       </c>
       <c r="D81" s="12">
-        <f>C81+C23+IF(B9="Armes de jet",10,0)</f>
-        <v/>
-      </c>
+        <f>C81+C23+IF($B$9="Armes de jet",10,0)</f>
+        <v/>
+      </c>
+      <c r="E81" s="26" t="n"/>
       <c r="F81" s="20" t="inlineStr">
         <is>
           <t>Négociation</t>
@@ -2636,6 +2803,7 @@
         <f>H81+H27</f>
         <v/>
       </c>
+      <c r="J81" s="26" t="n"/>
       <c r="K81" s="20" t="inlineStr">
         <is>
           <t>Géographie</t>
@@ -2655,12 +2823,12 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="22" t="inlineStr">
+      <c r="A82" s="20" t="inlineStr">
         <is>
           <t>Archerie</t>
         </is>
       </c>
-      <c r="B82" s="23" t="inlineStr">
+      <c r="B82" s="21" t="inlineStr">
         <is>
           <t>DEX</t>
         </is>
@@ -2669,15 +2837,16 @@
         <v>0</v>
       </c>
       <c r="D82" s="12">
-        <f>C82+C23+IF(B9="Archerie",10,0)</f>
-        <v/>
-      </c>
-      <c r="F82" s="22" t="inlineStr">
+        <f>C82+C23+IF($B$9="Archerie",10,0)</f>
+        <v/>
+      </c>
+      <c r="E82" s="26" t="n"/>
+      <c r="F82" s="20" t="inlineStr">
         <is>
           <t>Tromperie</t>
         </is>
       </c>
-      <c r="G82" s="23" t="inlineStr">
+      <c r="G82" s="21" t="inlineStr">
         <is>
           <t>CHA</t>
         </is>
@@ -2689,12 +2858,13 @@
         <f>H82+H27</f>
         <v/>
       </c>
-      <c r="K82" s="22" t="inlineStr">
+      <c r="J82" s="26" t="n"/>
+      <c r="K82" s="20" t="inlineStr">
         <is>
           <t>Cartographie</t>
         </is>
       </c>
-      <c r="L82" s="23" t="inlineStr">
+      <c r="L82" s="21" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
@@ -2722,9 +2892,10 @@
         <v>0</v>
       </c>
       <c r="D83" s="12">
-        <f>C83+C23+IF(B9="Armes à feu",10,0)</f>
-        <v/>
-      </c>
+        <f>C83+C23+IF($B$9="Armes à feu",10,0)</f>
+        <v/>
+      </c>
+      <c r="E83" s="26" t="n"/>
       <c r="F83" s="20" t="inlineStr">
         <is>
           <t>Séduction</t>
@@ -2732,16 +2903,17 @@
       </c>
       <c r="G83" s="21" t="inlineStr">
         <is>
-          <t>PRÉ</t>
+          <t>CHA</t>
         </is>
       </c>
       <c r="H83" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I83" s="12">
-        <f>H83+C27</f>
-        <v/>
-      </c>
+        <f>H83+H27</f>
+        <v/>
+      </c>
+      <c r="J83" s="26" t="n"/>
       <c r="K83" s="20" t="inlineStr">
         <is>
           <t>Économie</t>
@@ -2761,12 +2933,12 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="22" t="inlineStr">
+      <c r="A84" s="20" t="inlineStr">
         <is>
           <t>Parade</t>
         </is>
       </c>
-      <c r="B84" s="23" t="inlineStr">
+      <c r="B84" s="21" t="inlineStr">
         <is>
           <t>DEX</t>
         </is>
@@ -2775,15 +2947,16 @@
         <v>0</v>
       </c>
       <c r="D84" s="12">
-        <f>C84+C23+IF(G9="Parade",10,0)</f>
-        <v/>
-      </c>
-      <c r="F84" s="22" t="inlineStr">
+        <f>C84+C23+IF($G$9="Parade",10,0)</f>
+        <v/>
+      </c>
+      <c r="E84" s="26" t="n"/>
+      <c r="F84" s="20" t="inlineStr">
         <is>
           <t>Intimidation</t>
         </is>
       </c>
-      <c r="G84" s="23" t="inlineStr">
+      <c r="G84" s="21" t="inlineStr">
         <is>
           <t>PRÉ</t>
         </is>
@@ -2795,12 +2968,13 @@
         <f>H84+C27</f>
         <v/>
       </c>
-      <c r="K84" s="22" t="inlineStr">
+      <c r="J84" s="26" t="n"/>
+      <c r="K84" s="20" t="inlineStr">
         <is>
           <t>Estimation</t>
         </is>
       </c>
-      <c r="L84" s="23" t="inlineStr">
+      <c r="L84" s="21" t="inlineStr">
         <is>
           <t>ÉRU</t>
         </is>
@@ -2828,9 +3002,10 @@
         <v>0</v>
       </c>
       <c r="D85" s="12">
-        <f>C85+C24+IF(G9="Esquive",10,0)</f>
-        <v/>
-      </c>
+        <f>C85+C24+IF($G$9="Esquive",10,0)</f>
+        <v/>
+      </c>
+      <c r="E85" s="26" t="n"/>
       <c r="F85" s="20" t="inlineStr">
         <is>
           <t>Interrogatoire</t>
@@ -2848,6 +3023,7 @@
         <f>H85+H27</f>
         <v/>
       </c>
+      <c r="J85" s="26" t="n"/>
       <c r="K85" s="20" t="inlineStr">
         <is>
           <t>Politique</t>
@@ -2867,12 +3043,17 @@
       </c>
     </row>
     <row r="86">
-      <c r="F86" s="22" t="inlineStr">
+      <c r="A86" s="26" t="n"/>
+      <c r="B86" s="26" t="n"/>
+      <c r="C86" s="26" t="n"/>
+      <c r="D86" s="26" t="n"/>
+      <c r="E86" s="26" t="n"/>
+      <c r="F86" s="20" t="inlineStr">
         <is>
           <t>Commandement</t>
         </is>
       </c>
-      <c r="G86" s="23" t="inlineStr">
+      <c r="G86" s="21" t="inlineStr">
         <is>
           <t>PRÉ</t>
         </is>
@@ -2884,12 +3065,13 @@
         <f>H86+C27</f>
         <v/>
       </c>
-      <c r="K86" s="22" t="inlineStr">
+      <c r="J86" s="26" t="n"/>
+      <c r="K86" s="20" t="inlineStr">
         <is>
           <t>Droit</t>
         </is>
       </c>
-      <c r="L86" s="23" t="inlineStr">
+      <c r="L86" s="21" t="inlineStr">
         <is>
           <t>ÉRU</t>
         </is>
@@ -2908,9 +3090,10 @@
           <t>Champ Athlétique</t>
         </is>
       </c>
-      <c r="B87" s="6" t="n"/>
-      <c r="C87" s="6" t="n"/>
-      <c r="D87" s="6" t="n"/>
+      <c r="B87" s="9" t="n"/>
+      <c r="C87" s="9" t="n"/>
+      <c r="D87" s="10" t="n"/>
+      <c r="E87" s="26" t="n"/>
       <c r="F87" s="20" t="inlineStr">
         <is>
           <t>Pédagogie</t>
@@ -2918,16 +3101,17 @@
       </c>
       <c r="G87" s="21" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>ÉRU</t>
         </is>
       </c>
       <c r="H87" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I87" s="12">
-        <f>H87+H27</f>
-        <v/>
-      </c>
+        <f>H87+H25</f>
+        <v/>
+      </c>
+      <c r="J87" s="26" t="n"/>
       <c r="K87" s="20" t="inlineStr">
         <is>
           <t>Langues</t>
@@ -2967,12 +3151,13 @@
           <t>Bonus</t>
         </is>
       </c>
-      <c r="F88" s="22" t="inlineStr">
+      <c r="E88" s="26" t="n"/>
+      <c r="F88" s="20" t="inlineStr">
         <is>
           <t>Relation</t>
         </is>
       </c>
-      <c r="G88" s="23" t="inlineStr">
+      <c r="G88" s="21" t="inlineStr">
         <is>
           <t>CHA</t>
         </is>
@@ -2984,12 +3169,13 @@
         <f>H88+H27</f>
         <v/>
       </c>
-      <c r="K88" s="22" t="inlineStr">
+      <c r="J88" s="26" t="n"/>
+      <c r="K88" s="20" t="inlineStr">
         <is>
           <t>Astronomie</t>
         </is>
       </c>
-      <c r="L88" s="23" t="inlineStr">
+      <c r="L88" s="21" t="inlineStr">
         <is>
           <t>ÉRU</t>
         </is>
@@ -3020,6 +3206,7 @@
         <f>C89+C24</f>
         <v/>
       </c>
+      <c r="E89" s="26" t="n"/>
       <c r="F89" s="20" t="inlineStr">
         <is>
           <t>Étiquette</t>
@@ -3037,6 +3224,7 @@
         <f>H89+H25</f>
         <v/>
       </c>
+      <c r="J89" s="26" t="n"/>
       <c r="K89" s="20" t="inlineStr">
         <is>
           <t>Architecture</t>
@@ -3056,12 +3244,12 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="22" t="inlineStr">
+      <c r="A90" s="20" t="inlineStr">
         <is>
           <t>Saut</t>
         </is>
       </c>
-      <c r="B90" s="23" t="inlineStr">
+      <c r="B90" s="21" t="inlineStr">
         <is>
           <t>AGI</t>
         </is>
@@ -3073,12 +3261,13 @@
         <f>C90+C24</f>
         <v/>
       </c>
-      <c r="F90" s="22" t="inlineStr">
+      <c r="E90" s="26" t="n"/>
+      <c r="F90" s="20" t="inlineStr">
         <is>
           <t>Style</t>
         </is>
       </c>
-      <c r="G90" s="23" t="inlineStr">
+      <c r="G90" s="21" t="inlineStr">
         <is>
           <t>PRÉ</t>
         </is>
@@ -3090,12 +3279,13 @@
         <f>H90+C27</f>
         <v/>
       </c>
-      <c r="K90" s="22" t="inlineStr">
+      <c r="J90" s="26" t="n"/>
+      <c r="K90" s="20" t="inlineStr">
         <is>
           <t>Géologie</t>
         </is>
       </c>
-      <c r="L90" s="23" t="inlineStr">
+      <c r="L90" s="21" t="inlineStr">
         <is>
           <t>ÉRU</t>
         </is>
@@ -3126,9 +3316,15 @@
         <f>C91+C24</f>
         <v/>
       </c>
+      <c r="E91" s="26" t="n"/>
+      <c r="F91" s="26" t="n"/>
+      <c r="G91" s="26" t="n"/>
+      <c r="H91" s="26" t="n"/>
+      <c r="I91" s="26" t="n"/>
+      <c r="J91" s="26" t="n"/>
       <c r="K91" s="20" t="inlineStr">
         <is>
-          <t>Faune</t>
+          <t>Biologie</t>
         </is>
       </c>
       <c r="L91" s="21" t="inlineStr">
@@ -3145,37 +3341,39 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="22" t="inlineStr">
+      <c r="A92" s="20" t="inlineStr">
         <is>
           <t>Escalade</t>
         </is>
       </c>
-      <c r="B92" s="23" t="inlineStr">
-        <is>
-          <t>FOR</t>
+      <c r="B92" s="21" t="inlineStr">
+        <is>
+          <t>AGI</t>
         </is>
       </c>
       <c r="C92" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D92" s="12">
-        <f>C92+C22</f>
-        <v/>
-      </c>
+        <f>C92+C24</f>
+        <v/>
+      </c>
+      <c r="E92" s="26" t="n"/>
       <c r="F92" s="19" t="inlineStr">
         <is>
-          <t>Champ Sauvage</t>
-        </is>
-      </c>
-      <c r="G92" s="6" t="n"/>
-      <c r="H92" s="6" t="n"/>
-      <c r="I92" s="6" t="n"/>
-      <c r="K92" s="22" t="inlineStr">
-        <is>
-          <t>Flore</t>
-        </is>
-      </c>
-      <c r="L92" s="23" t="inlineStr">
+          <t>Champ Naturel</t>
+        </is>
+      </c>
+      <c r="G92" s="9" t="n"/>
+      <c r="H92" s="9" t="n"/>
+      <c r="I92" s="10" t="n"/>
+      <c r="J92" s="26" t="n"/>
+      <c r="K92" s="20" t="inlineStr">
+        <is>
+          <t>Faune</t>
+        </is>
+      </c>
+      <c r="L92" s="21" t="inlineStr">
         <is>
           <t>ÉRU</t>
         </is>
@@ -3206,6 +3404,7 @@
         <f>C93+C24</f>
         <v/>
       </c>
+      <c r="E93" s="26" t="n"/>
       <c r="F93" s="14" t="inlineStr">
         <is>
           <t>Compétence</t>
@@ -3226,31 +3425,32 @@
           <t>Bonus</t>
         </is>
       </c>
+      <c r="J93" s="26" t="n"/>
       <c r="K93" s="20" t="inlineStr">
         <is>
-          <t>Météorologie</t>
+          <t>Flore</t>
         </is>
       </c>
       <c r="L93" s="21" t="inlineStr">
         <is>
-          <t>INS</t>
+          <t>ÉRU</t>
         </is>
       </c>
       <c r="M93" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N93" s="12">
-        <f>M93+H24</f>
+        <f>M93+H25</f>
         <v/>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="22" t="inlineStr">
+      <c r="A94" s="20" t="inlineStr">
         <is>
           <t>Contorsion</t>
         </is>
       </c>
-      <c r="B94" s="23" t="inlineStr">
+      <c r="B94" s="21" t="inlineStr">
         <is>
           <t>AGI</t>
         </is>
@@ -3262,6 +3462,7 @@
         <f>C94+C24</f>
         <v/>
       </c>
+      <c r="E94" s="26" t="n"/>
       <c r="F94" s="20" t="inlineStr">
         <is>
           <t>Survie</t>
@@ -3279,12 +3480,13 @@
         <f>H94+H24</f>
         <v/>
       </c>
-      <c r="K94" s="22" t="inlineStr">
-        <is>
-          <t>Mémorisation</t>
-        </is>
-      </c>
-      <c r="L94" s="23" t="inlineStr">
+      <c r="J94" s="26" t="n"/>
+      <c r="K94" s="20" t="inlineStr">
+        <is>
+          <t>Météorologie</t>
+        </is>
+      </c>
+      <c r="L94" s="21" t="inlineStr">
         <is>
           <t>ÉRU</t>
         </is>
@@ -3315,12 +3517,13 @@
         <f>C95+C24</f>
         <v/>
       </c>
-      <c r="F95" s="22" t="inlineStr">
+      <c r="E95" s="26" t="n"/>
+      <c r="F95" s="20" t="inlineStr">
         <is>
           <t>Pistage</t>
         </is>
       </c>
-      <c r="G95" s="23" t="inlineStr">
+      <c r="G95" s="21" t="inlineStr">
         <is>
           <t>INS</t>
         </is>
@@ -3332,9 +3535,10 @@
         <f>H95+H24</f>
         <v/>
       </c>
+      <c r="J95" s="26" t="n"/>
       <c r="K95" s="20" t="inlineStr">
         <is>
-          <t>Occultisme</t>
+          <t>Mémorisation</t>
         </is>
       </c>
       <c r="L95" s="21" t="inlineStr">
@@ -3351,12 +3555,12 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="22" t="inlineStr">
+      <c r="A96" s="20" t="inlineStr">
         <is>
           <t>Lutte</t>
         </is>
       </c>
-      <c r="B96" s="23" t="inlineStr">
+      <c r="B96" s="21" t="inlineStr">
         <is>
           <t>FOR</t>
         </is>
@@ -3368,6 +3572,7 @@
         <f>C96+C22+10</f>
         <v/>
       </c>
+      <c r="E96" s="26" t="n"/>
       <c r="F96" s="20" t="inlineStr">
         <is>
           <t>Chasse</t>
@@ -3385,12 +3590,13 @@
         <f>H96+H24</f>
         <v/>
       </c>
-      <c r="K96" s="22" t="inlineStr">
-        <is>
-          <t>Théologie</t>
-        </is>
-      </c>
-      <c r="L96" s="23" t="inlineStr">
+      <c r="J96" s="26" t="n"/>
+      <c r="K96" s="20" t="inlineStr">
+        <is>
+          <t>Occultisme</t>
+        </is>
+      </c>
+      <c r="L96" s="21" t="inlineStr">
         <is>
           <t>ÉRU</t>
         </is>
@@ -3421,12 +3627,13 @@
         <f>C97+C22</f>
         <v/>
       </c>
-      <c r="F97" s="22" t="inlineStr">
+      <c r="E97" s="26" t="n"/>
+      <c r="F97" s="20" t="inlineStr">
         <is>
           <t>Pêche</t>
         </is>
       </c>
-      <c r="G97" s="23" t="inlineStr">
+      <c r="G97" s="21" t="inlineStr">
         <is>
           <t>INS</t>
         </is>
@@ -3438,9 +3645,10 @@
         <f>H97+H24</f>
         <v/>
       </c>
+      <c r="J97" s="26" t="n"/>
       <c r="K97" s="20" t="inlineStr">
         <is>
-          <t>Médecine</t>
+          <t>Théologie</t>
         </is>
       </c>
       <c r="L97" s="21" t="inlineStr">
@@ -3457,12 +3665,12 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="22" t="inlineStr">
+      <c r="A98" s="20" t="inlineStr">
         <is>
           <t>Apnée</t>
         </is>
       </c>
-      <c r="B98" s="23" t="inlineStr">
+      <c r="B98" s="21" t="inlineStr">
         <is>
           <t>END</t>
         </is>
@@ -3474,6 +3682,7 @@
         <f>C98+C25</f>
         <v/>
       </c>
+      <c r="E98" s="26" t="n"/>
       <c r="F98" s="20" t="inlineStr">
         <is>
           <t>Dressage</t>
@@ -3491,57 +3700,64 @@
         <f>H98+H24</f>
         <v/>
       </c>
-      <c r="K98" s="22" t="inlineStr">
+      <c r="J98" s="26" t="n"/>
+      <c r="K98" s="20" t="inlineStr">
+        <is>
+          <t>Médecine</t>
+        </is>
+      </c>
+      <c r="L98" s="21" t="inlineStr">
+        <is>
+          <t>ÉRU</t>
+        </is>
+      </c>
+      <c r="M98" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N98" s="12">
+        <f>M98+H25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="26" t="n"/>
+      <c r="B99" s="26" t="n"/>
+      <c r="C99" s="26" t="n"/>
+      <c r="D99" s="26" t="n"/>
+      <c r="E99" s="26" t="n"/>
+      <c r="F99" s="20" t="inlineStr">
+        <is>
+          <t>Élevage</t>
+        </is>
+      </c>
+      <c r="G99" s="21" t="inlineStr">
+        <is>
+          <t>ÉRU</t>
+        </is>
+      </c>
+      <c r="H99" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" s="12">
+        <f>H99+H25</f>
+        <v/>
+      </c>
+      <c r="J99" s="26" t="n"/>
+      <c r="K99" s="20" t="inlineStr">
         <is>
           <t>Enquête</t>
         </is>
       </c>
-      <c r="L98" s="23" t="inlineStr">
+      <c r="L99" s="21" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="M98" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N98" s="12">
-        <f>M98+H23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99">
-      <c r="F99" s="22" t="inlineStr">
-        <is>
-          <t>Élevage</t>
-        </is>
-      </c>
-      <c r="G99" s="23" t="inlineStr">
-        <is>
-          <t>INS</t>
-        </is>
-      </c>
-      <c r="H99" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I99" s="12">
-        <f>H99+H24</f>
-        <v/>
-      </c>
-      <c r="K99" s="20" t="inlineStr">
-        <is>
-          <t>Psychologie</t>
-        </is>
-      </c>
-      <c r="L99" s="21" t="inlineStr">
-        <is>
-          <t>ÉRU</t>
-        </is>
-      </c>
       <c r="M99" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N99" s="12">
-        <f>M99+H25</f>
+        <f>M99+H23</f>
         <v/>
       </c>
     </row>
@@ -3551,9 +3767,10 @@
           <t>Champ Vital</t>
         </is>
       </c>
-      <c r="B100" s="6" t="n"/>
-      <c r="C100" s="6" t="n"/>
-      <c r="D100" s="6" t="n"/>
+      <c r="B100" s="9" t="n"/>
+      <c r="C100" s="9" t="n"/>
+      <c r="D100" s="10" t="n"/>
+      <c r="E100" s="26" t="n"/>
       <c r="F100" s="20" t="inlineStr">
         <is>
           <t>Agriculture</t>
@@ -3561,31 +3778,32 @@
       </c>
       <c r="G100" s="21" t="inlineStr">
         <is>
-          <t>INS</t>
+          <t>ÉRU</t>
         </is>
       </c>
       <c r="H100" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I100" s="12">
-        <f>H100+H24</f>
-        <v/>
-      </c>
-      <c r="K100" s="22" t="inlineStr">
-        <is>
-          <t>Perspicacité</t>
-        </is>
-      </c>
-      <c r="L100" s="23" t="inlineStr">
-        <is>
-          <t>INS</t>
+        <f>H100+H25</f>
+        <v/>
+      </c>
+      <c r="J100" s="26" t="n"/>
+      <c r="K100" s="20" t="inlineStr">
+        <is>
+          <t>Psychologie</t>
+        </is>
+      </c>
+      <c r="L100" s="21" t="inlineStr">
+        <is>
+          <t>ÉRU</t>
         </is>
       </c>
       <c r="M100" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N100" s="12">
-        <f>M100+H24</f>
+        <f>M100+H25</f>
         <v/>
       </c>
     </row>
@@ -3610,21 +3828,27 @@
           <t>Bonus</t>
         </is>
       </c>
+      <c r="E101" s="26" t="n"/>
+      <c r="F101" s="26" t="n"/>
+      <c r="G101" s="26" t="n"/>
+      <c r="H101" s="26" t="n"/>
+      <c r="I101" s="26" t="n"/>
+      <c r="J101" s="26" t="n"/>
       <c r="K101" s="20" t="inlineStr">
         <is>
-          <t>Tactique</t>
+          <t>Perspicacité</t>
         </is>
       </c>
       <c r="L101" s="21" t="inlineStr">
         <is>
-          <t>LOG</t>
+          <t>INS</t>
         </is>
       </c>
       <c r="M101" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N101" s="12">
-        <f>M101+H23</f>
+        <f>M101+H24</f>
         <v/>
       </c>
     </row>
@@ -3646,20 +3870,22 @@
         <f>C102+C25</f>
         <v/>
       </c>
+      <c r="E102" s="26" t="n"/>
       <c r="F102" s="19" t="inlineStr">
         <is>
-          <t>Champ Technique</t>
-        </is>
-      </c>
-      <c r="G102" s="6" t="n"/>
-      <c r="H102" s="6" t="n"/>
-      <c r="I102" s="6" t="n"/>
-      <c r="K102" s="22" t="inlineStr">
-        <is>
-          <t>Jeu d'argent</t>
-        </is>
-      </c>
-      <c r="L102" s="23" t="inlineStr">
+          <t>Champ Artisanal</t>
+        </is>
+      </c>
+      <c r="G102" s="9" t="n"/>
+      <c r="H102" s="9" t="n"/>
+      <c r="I102" s="10" t="n"/>
+      <c r="J102" s="26" t="n"/>
+      <c r="K102" s="20" t="inlineStr">
+        <is>
+          <t>Tactique</t>
+        </is>
+      </c>
+      <c r="L102" s="21" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
@@ -3673,12 +3899,12 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="22" t="inlineStr">
+      <c r="A103" s="20" t="inlineStr">
         <is>
           <t>Résistance aux Toxines</t>
         </is>
       </c>
-      <c r="B103" s="23" t="inlineStr">
+      <c r="B103" s="21" t="inlineStr">
         <is>
           <t>END</t>
         </is>
@@ -3690,6 +3916,7 @@
         <f>C103+C25</f>
         <v/>
       </c>
+      <c r="E103" s="26" t="n"/>
       <c r="F103" s="14" t="inlineStr">
         <is>
           <t>Compétence</t>
@@ -3710,9 +3937,10 @@
           <t>Bonus</t>
         </is>
       </c>
+      <c r="J103" s="26" t="n"/>
       <c r="K103" s="20" t="inlineStr">
         <is>
-          <t>Jeux de stratégie</t>
+          <t>Jeu d'argent</t>
         </is>
       </c>
       <c r="L103" s="21" t="inlineStr">
@@ -3736,41 +3964,60 @@
       </c>
       <c r="B104" s="21" t="inlineStr">
         <is>
-          <t>END</t>
+          <t>VOL</t>
         </is>
       </c>
       <c r="C104" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D104" s="12">
-        <f>C104+C25+10</f>
-        <v/>
-      </c>
+        <f>C104+H22+10</f>
+        <v/>
+      </c>
+      <c r="E104" s="26" t="n"/>
       <c r="F104" s="20" t="inlineStr">
         <is>
-          <t>Mécanique</t>
+          <t>Forge / Métallurgie</t>
         </is>
       </c>
       <c r="G104" s="21" t="inlineStr">
         <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="H104" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I104" s="12">
+        <f>H104+C23</f>
+        <v/>
+      </c>
+      <c r="J104" s="26" t="n"/>
+      <c r="K104" s="20" t="inlineStr">
+        <is>
+          <t>Jeux de stratégie</t>
+        </is>
+      </c>
+      <c r="L104" s="21" t="inlineStr">
+        <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="H104" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I104" s="12">
-        <f>H104+H23</f>
+      <c r="M104" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N104" s="12">
+        <f>M104+H23</f>
         <v/>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="22" t="inlineStr">
+      <c r="A105" s="20" t="inlineStr">
         <is>
           <t>Résistance à l'Environnement</t>
         </is>
       </c>
-      <c r="B105" s="23" t="inlineStr">
+      <c r="B105" s="21" t="inlineStr">
         <is>
           <t>END</t>
         </is>
@@ -3782,426 +4029,449 @@
         <f>C105+C25</f>
         <v/>
       </c>
-      <c r="F105" s="22" t="inlineStr">
-        <is>
-          <t>Électronique</t>
-        </is>
-      </c>
-      <c r="G105" s="23" t="inlineStr">
-        <is>
-          <t>LOG</t>
+      <c r="E105" s="26" t="n"/>
+      <c r="F105" s="20" t="inlineStr">
+        <is>
+          <t>Travail du bois</t>
+        </is>
+      </c>
+      <c r="G105" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
         </is>
       </c>
       <c r="H105" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I105" s="12">
-        <f>H105+H23</f>
-        <v/>
-      </c>
-      <c r="K105" s="19" t="inlineStr">
-        <is>
-          <t>Champ Sensoriel (13 sens)</t>
-        </is>
-      </c>
-      <c r="L105" s="6" t="n"/>
-      <c r="M105" s="6" t="n"/>
-      <c r="N105" s="6" t="n"/>
+        <f>H105+C23</f>
+        <v/>
+      </c>
+      <c r="J105" s="26" t="n"/>
+      <c r="K105" s="27" t="n"/>
+      <c r="L105" s="26" t="n"/>
+      <c r="M105" s="26" t="n"/>
+      <c r="N105" s="26" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="20" t="inlineStr">
         <is>
+          <t>Résistance à la Fatigue</t>
+        </is>
+      </c>
+      <c r="B106" s="21" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="C106" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" s="12">
+        <f>C106+C25</f>
+        <v/>
+      </c>
+      <c r="E106" s="26" t="n"/>
+      <c r="F106" s="20" t="inlineStr">
+        <is>
+          <t>Travail de la pierre</t>
+        </is>
+      </c>
+      <c r="G106" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="H106" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" s="12">
+        <f>H106+C23</f>
+        <v/>
+      </c>
+      <c r="J106" s="26" t="n"/>
+      <c r="K106" s="19" t="inlineStr">
+        <is>
+          <t>Champ Sensoriel</t>
+        </is>
+      </c>
+      <c r="L106" s="9" t="n"/>
+      <c r="M106" s="9" t="n"/>
+      <c r="N106" s="10" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="20" t="inlineStr">
+        <is>
           <t>Résistance Mentale</t>
         </is>
       </c>
-      <c r="B106" s="21" t="inlineStr">
+      <c r="B107" s="21" t="inlineStr">
         <is>
           <t>VOL</t>
         </is>
       </c>
-      <c r="C106" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D106" s="12">
-        <f>C106+H22</f>
-        <v/>
-      </c>
-      <c r="F106" s="20" t="inlineStr">
-        <is>
-          <t>Programmation</t>
-        </is>
-      </c>
-      <c r="G106" s="21" t="inlineStr">
-        <is>
-          <t>LOG</t>
-        </is>
-      </c>
-      <c r="H106" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I106" s="12">
-        <f>H106+H23</f>
-        <v/>
-      </c>
-      <c r="K106" s="14" t="inlineStr">
-        <is>
-          <t>Sens</t>
-        </is>
-      </c>
-      <c r="L106" s="14" t="inlineStr">
-        <is>
-          <t>Acuité</t>
-        </is>
-      </c>
-      <c r="M106" s="14" t="inlineStr">
+      <c r="C107" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="12">
+        <f>C107+H22</f>
+        <v/>
+      </c>
+      <c r="E107" s="26" t="n"/>
+      <c r="F107" s="20" t="inlineStr">
+        <is>
+          <t>Textile</t>
+        </is>
+      </c>
+      <c r="G107" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="H107" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" s="12">
+        <f>H107+C23</f>
+        <v/>
+      </c>
+      <c r="J107" s="26" t="n"/>
+      <c r="K107" s="14" t="inlineStr">
+        <is>
+          <t>Compétence</t>
+        </is>
+      </c>
+      <c r="L107" s="14" t="inlineStr">
+        <is>
+          <t>Carac</t>
+        </is>
+      </c>
+      <c r="M107" s="14" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="N106" s="14" t="inlineStr">
-        <is>
-          <t>Bonus / Malus</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="F107" s="22" t="inlineStr">
-        <is>
-          <t>Cybersécurité</t>
-        </is>
-      </c>
-      <c r="G107" s="23" t="inlineStr">
-        <is>
-          <t>LOG</t>
-        </is>
-      </c>
-      <c r="H107" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I107" s="12">
-        <f>H107+H23</f>
-        <v/>
-      </c>
-      <c r="K107" s="20" t="inlineStr">
-        <is>
-          <t>Observation / Vue</t>
-        </is>
-      </c>
-      <c r="L107" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="M107" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N107" s="12">
-        <f>(10-L107)*-20</f>
-        <v/>
+      <c r="N107" s="14" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="19" t="inlineStr">
+      <c r="A108" s="27" t="n"/>
+      <c r="B108" s="26" t="n"/>
+      <c r="C108" s="26" t="n"/>
+      <c r="D108" s="26" t="n"/>
+      <c r="E108" s="26" t="n"/>
+      <c r="F108" s="20" t="inlineStr">
+        <is>
+          <t>Travail du cuir</t>
+        </is>
+      </c>
+      <c r="G108" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="H108" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" s="12">
+        <f>H108+C23</f>
+        <v/>
+      </c>
+      <c r="J108" s="26" t="n"/>
+      <c r="K108" s="20" t="inlineStr">
+        <is>
+          <t>Vue</t>
+        </is>
+      </c>
+      <c r="L108" s="21" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="M108" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" s="12">
+        <f>M108+C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="19" t="inlineStr">
         <is>
           <t>Champ Furtif</t>
         </is>
       </c>
-      <c r="B108" s="6" t="n"/>
-      <c r="C108" s="6" t="n"/>
-      <c r="D108" s="6" t="n"/>
-      <c r="F108" s="20" t="inlineStr">
-        <is>
-          <t>Réseaux &amp; télécoms</t>
-        </is>
-      </c>
-      <c r="G108" s="21" t="inlineStr">
-        <is>
-          <t>LOG</t>
-        </is>
-      </c>
-      <c r="H108" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I108" s="12">
-        <f>H108+H23</f>
-        <v/>
-      </c>
-      <c r="K108" s="22" t="inlineStr">
+      <c r="B109" s="9" t="n"/>
+      <c r="C109" s="9" t="n"/>
+      <c r="D109" s="10" t="n"/>
+      <c r="E109" s="26" t="n"/>
+      <c r="F109" s="20" t="inlineStr">
+        <is>
+          <t>Poterie</t>
+        </is>
+      </c>
+      <c r="G109" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="H109" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" s="12">
+        <f>H109+C23</f>
+        <v/>
+      </c>
+      <c r="J109" s="26" t="n"/>
+      <c r="K109" s="20" t="inlineStr">
         <is>
           <t>Ouïe</t>
         </is>
       </c>
-      <c r="L108" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="M108" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N108" s="12">
-        <f>(10-L108)*-20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="14" t="inlineStr">
+      <c r="L109" s="21" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="M109" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N109" s="12">
+        <f>M109+C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="inlineStr">
         <is>
           <t>Compétence</t>
         </is>
       </c>
-      <c r="B109" s="14" t="inlineStr">
+      <c r="B110" s="14" t="inlineStr">
         <is>
           <t>Carac</t>
         </is>
       </c>
-      <c r="C109" s="14" t="inlineStr">
+      <c r="C110" s="14" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="D109" s="14" t="inlineStr">
+      <c r="D110" s="14" t="inlineStr">
         <is>
           <t>Bonus</t>
         </is>
       </c>
-      <c r="F109" s="22" t="inlineStr">
-        <is>
-          <t>Cryptographie</t>
-        </is>
-      </c>
-      <c r="G109" s="23" t="inlineStr">
-        <is>
-          <t>LOG</t>
-        </is>
-      </c>
-      <c r="H109" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I109" s="12">
-        <f>H109+H23</f>
-        <v/>
-      </c>
-      <c r="K109" s="20" t="inlineStr">
+      <c r="E110" s="26" t="n"/>
+      <c r="F110" s="20" t="inlineStr">
+        <is>
+          <t>Verre</t>
+        </is>
+      </c>
+      <c r="G110" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="H110" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" s="12">
+        <f>H110+C23</f>
+        <v/>
+      </c>
+      <c r="J110" s="26" t="n"/>
+      <c r="K110" s="20" t="inlineStr">
         <is>
           <t>Odorat</t>
         </is>
       </c>
-      <c r="L109" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="M109" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N109" s="12">
-        <f>(10-L109)*-20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="20" t="inlineStr">
+      <c r="L110" s="21" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="M110" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N110" s="12">
+        <f>M110+C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="20" t="inlineStr">
         <is>
           <t>Discrétion</t>
         </is>
       </c>
-      <c r="B110" s="21" t="inlineStr">
+      <c r="B111" s="21" t="inlineStr">
         <is>
           <t>AGI</t>
         </is>
       </c>
-      <c r="C110" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D110" s="12">
-        <f>C110+C24</f>
-        <v/>
-      </c>
-      <c r="F110" s="20" t="inlineStr">
-        <is>
-          <t>Chimie</t>
-        </is>
-      </c>
-      <c r="G110" s="21" t="inlineStr">
-        <is>
-          <t>LOG</t>
-        </is>
-      </c>
-      <c r="H110" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I110" s="12">
-        <f>H110+H23</f>
-        <v/>
-      </c>
-      <c r="K110" s="22" t="inlineStr">
+      <c r="C111" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" s="12">
+        <f>C111+C24</f>
+        <v/>
+      </c>
+      <c r="E111" s="26" t="n"/>
+      <c r="F111" s="20" t="inlineStr">
+        <is>
+          <t>Joaillerie</t>
+        </is>
+      </c>
+      <c r="G111" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="H111" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" s="12">
+        <f>H111+C23</f>
+        <v/>
+      </c>
+      <c r="J111" s="26" t="n"/>
+      <c r="K111" s="20" t="inlineStr">
         <is>
           <t>Goût</t>
         </is>
       </c>
-      <c r="L110" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="M110" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N110" s="12">
-        <f>(10-L110)*-20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="22" t="inlineStr">
-        <is>
-          <t>Camouflage</t>
-        </is>
-      </c>
-      <c r="B111" s="23" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
-      <c r="C111" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D111" s="12">
-        <f>C111+C23</f>
-        <v/>
-      </c>
-      <c r="F111" s="22" t="inlineStr">
-        <is>
-          <t>Pharmacologie</t>
-        </is>
-      </c>
-      <c r="G111" s="23" t="inlineStr">
-        <is>
-          <t>LOG</t>
-        </is>
-      </c>
-      <c r="H111" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I111" s="12">
-        <f>H111+H23</f>
-        <v/>
-      </c>
-      <c r="K111" s="20" t="inlineStr">
-        <is>
-          <t>Toucher</t>
-        </is>
-      </c>
-      <c r="L111" s="11" t="n">
-        <v>10</v>
+      <c r="L111" s="21" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
       </c>
       <c r="M111" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N111" s="12">
-        <f>(10-L111)*-20</f>
+        <f>M111+C26</f>
         <v/>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="20" t="inlineStr">
         <is>
+          <t>Camouflage</t>
+        </is>
+      </c>
+      <c r="B112" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" s="12">
+        <f>C112+C23</f>
+        <v/>
+      </c>
+      <c r="E112" s="26" t="n"/>
+      <c r="F112" s="20" t="inlineStr">
+        <is>
+          <t>Cuisine</t>
+        </is>
+      </c>
+      <c r="G112" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="H112" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" s="12">
+        <f>H112+C23</f>
+        <v/>
+      </c>
+      <c r="J112" s="26" t="n"/>
+      <c r="K112" s="20" t="inlineStr">
+        <is>
+          <t>Toucher</t>
+        </is>
+      </c>
+      <c r="L112" s="21" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="M112" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" s="12">
+        <f>M112+C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="20" t="inlineStr">
+        <is>
           <t>Filature</t>
         </is>
       </c>
-      <c r="B112" s="21" t="inlineStr">
+      <c r="B113" s="21" t="inlineStr">
         <is>
           <t>PER</t>
         </is>
       </c>
-      <c r="C112" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D112" s="12">
-        <f>C112+C26</f>
-        <v/>
-      </c>
-      <c r="F112" s="20" t="inlineStr">
-        <is>
-          <t>Explosifs</t>
-        </is>
-      </c>
-      <c r="G112" s="21" t="inlineStr">
-        <is>
-          <t>LOG</t>
-        </is>
-      </c>
-      <c r="H112" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I112" s="12">
-        <f>H112+H23</f>
-        <v/>
-      </c>
-      <c r="K112" s="22" t="inlineStr">
-        <is>
-          <t>Chémoréception</t>
-        </is>
-      </c>
-      <c r="L112" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="M112" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N112" s="12">
-        <f>(10-L112)*-20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="22" t="inlineStr">
-        <is>
-          <t>Escamotage</t>
-        </is>
-      </c>
-      <c r="B113" s="23" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
       <c r="C113" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D113" s="12">
-        <f>C113+C23</f>
-        <v/>
-      </c>
-      <c r="F113" s="22" t="inlineStr">
-        <is>
-          <t>Conduite</t>
-        </is>
-      </c>
-      <c r="G113" s="23" t="inlineStr">
-        <is>
-          <t>AGI</t>
+        <f>C113+C26</f>
+        <v/>
+      </c>
+      <c r="E113" s="26" t="n"/>
+      <c r="F113" s="20" t="inlineStr">
+        <is>
+          <t>Brasserie &amp; distillation</t>
+        </is>
+      </c>
+      <c r="G113" s="21" t="inlineStr">
+        <is>
+          <t>ÉRU</t>
         </is>
       </c>
       <c r="H113" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I113" s="12">
-        <f>H113+C24</f>
-        <v/>
-      </c>
+        <f>H113+H25</f>
+        <v/>
+      </c>
+      <c r="J113" s="26" t="n"/>
       <c r="K113" s="20" t="inlineStr">
         <is>
-          <t>Chronoception</t>
-        </is>
-      </c>
-      <c r="L113" s="11" t="n">
-        <v>10</v>
+          <t>Chémesthésie</t>
+        </is>
+      </c>
+      <c r="L113" s="21" t="inlineStr">
+        <is>
+          <t>INS</t>
+        </is>
       </c>
       <c r="M113" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N113" s="12">
-        <f>(10-L113)*-20</f>
+        <f>M113+H24</f>
         <v/>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="20" t="inlineStr">
         <is>
-          <t>Crochetage</t>
+          <t>Escamotage</t>
         </is>
       </c>
       <c r="B114" s="21" t="inlineStr">
@@ -4216,46 +4486,50 @@
         <f>C114+C23</f>
         <v/>
       </c>
+      <c r="E114" s="26" t="n"/>
       <c r="F114" s="20" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Parfumerie</t>
         </is>
       </c>
       <c r="G114" s="21" t="inlineStr">
         <is>
-          <t>AGI</t>
+          <t>ÉRU</t>
         </is>
       </c>
       <c r="H114" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I114" s="12">
-        <f>H114+C24</f>
-        <v/>
-      </c>
-      <c r="K114" s="22" t="inlineStr">
-        <is>
-          <t>Équilibrioception</t>
-        </is>
-      </c>
-      <c r="L114" s="11" t="n">
-        <v>10</v>
+        <f>H114+H25</f>
+        <v/>
+      </c>
+      <c r="J114" s="26" t="n"/>
+      <c r="K114" s="20" t="inlineStr">
+        <is>
+          <t>Chronoception</t>
+        </is>
+      </c>
+      <c r="L114" s="21" t="inlineStr">
+        <is>
+          <t>INS</t>
+        </is>
       </c>
       <c r="M114" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N114" s="12">
-        <f>(10-L114)*-20</f>
+        <f>M114+H24</f>
         <v/>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="22" t="inlineStr">
-        <is>
-          <t>Pièges</t>
-        </is>
-      </c>
-      <c r="B115" s="23" t="inlineStr">
+      <c r="A115" s="20" t="inlineStr">
+        <is>
+          <t>Crochetage</t>
+        </is>
+      </c>
+      <c r="B115" s="21" t="inlineStr">
         <is>
           <t>DEX</t>
         </is>
@@ -4267,43 +4541,47 @@
         <f>C115+C23</f>
         <v/>
       </c>
-      <c r="F115" s="22" t="inlineStr">
-        <is>
-          <t>Pilotage</t>
-        </is>
-      </c>
-      <c r="G115" s="23" t="inlineStr">
-        <is>
-          <t>AGI</t>
+      <c r="E115" s="26" t="n"/>
+      <c r="F115" s="20" t="inlineStr">
+        <is>
+          <t>Calligraphie</t>
+        </is>
+      </c>
+      <c r="G115" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
         </is>
       </c>
       <c r="H115" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I115" s="12">
-        <f>H115+C24</f>
-        <v/>
-      </c>
+        <f>H115+C23</f>
+        <v/>
+      </c>
+      <c r="J115" s="26" t="n"/>
       <c r="K115" s="20" t="inlineStr">
         <is>
-          <t>Intéroception</t>
-        </is>
-      </c>
-      <c r="L115" s="11" t="n">
-        <v>10</v>
+          <t>Équilibrioception</t>
+        </is>
+      </c>
+      <c r="L115" s="21" t="inlineStr">
+        <is>
+          <t>INS</t>
+        </is>
       </c>
       <c r="M115" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N115" s="12">
-        <f>(10-L115)*-20</f>
+        <f>M115+H24</f>
         <v/>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="20" t="inlineStr">
         <is>
-          <t>Déguisement</t>
+          <t>Pièges</t>
         </is>
       </c>
       <c r="B116" s="21" t="inlineStr">
@@ -4318,46 +4596,37 @@
         <f>C116+C23</f>
         <v/>
       </c>
-      <c r="F116" s="20" t="inlineStr">
-        <is>
-          <t>Équitation</t>
-        </is>
-      </c>
-      <c r="G116" s="21" t="inlineStr">
-        <is>
-          <t>AGI</t>
-        </is>
-      </c>
-      <c r="H116" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I116" s="12">
-        <f>H116+C24</f>
-        <v/>
-      </c>
-      <c r="K116" s="22" t="inlineStr">
-        <is>
-          <t>Magnétoréception</t>
-        </is>
-      </c>
-      <c r="L116" s="11" t="n">
-        <v>10</v>
+      <c r="E116" s="26" t="n"/>
+      <c r="F116" s="27" t="n"/>
+      <c r="G116" s="28" t="n"/>
+      <c r="H116" s="28" t="n"/>
+      <c r="I116" s="28" t="n"/>
+      <c r="J116" s="26" t="n"/>
+      <c r="K116" s="20" t="inlineStr">
+        <is>
+          <t>Intéroception</t>
+        </is>
+      </c>
+      <c r="L116" s="21" t="inlineStr">
+        <is>
+          <t>INS</t>
+        </is>
       </c>
       <c r="M116" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N116" s="12">
-        <f>(10-L116)*-20</f>
+        <f>M116+H24</f>
         <v/>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="22" t="inlineStr">
-        <is>
-          <t>Contrefaçon</t>
-        </is>
-      </c>
-      <c r="B117" s="23" t="inlineStr">
+      <c r="A117" s="20" t="inlineStr">
+        <is>
+          <t>Déguisement</t>
+        </is>
+      </c>
+      <c r="B117" s="21" t="inlineStr">
         <is>
           <t>DEX</t>
         </is>
@@ -4369,430 +4638,766 @@
         <f>C117+C23</f>
         <v/>
       </c>
+      <c r="E117" s="26" t="n"/>
+      <c r="F117" s="19" t="inlineStr">
+        <is>
+          <t>Champ Artistique</t>
+        </is>
+      </c>
+      <c r="G117" s="9" t="n"/>
+      <c r="H117" s="9" t="n"/>
+      <c r="I117" s="10" t="n"/>
+      <c r="J117" s="26" t="n"/>
       <c r="K117" s="20" t="inlineStr">
         <is>
           <t>Nociception</t>
         </is>
       </c>
-      <c r="L117" s="11" t="n">
-        <v>10</v>
+      <c r="L117" s="21" t="inlineStr">
+        <is>
+          <t>INS</t>
+        </is>
       </c>
       <c r="M117" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N117" s="12">
-        <f>(10-L117)*-20</f>
+        <f>M117+H24</f>
         <v/>
       </c>
     </row>
     <row r="118">
-      <c r="F118" s="19" t="inlineStr">
-        <is>
-          <t>Champ Créatif</t>
-        </is>
-      </c>
-      <c r="G118" s="6" t="n"/>
-      <c r="H118" s="6" t="n"/>
-      <c r="I118" s="6" t="n"/>
-      <c r="K118" s="22" t="inlineStr">
+      <c r="A118" s="20" t="inlineStr">
+        <is>
+          <t>Contrefaçon</t>
+        </is>
+      </c>
+      <c r="B118" s="21" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="C118" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" s="12">
+        <f>C118+C23</f>
+        <v/>
+      </c>
+      <c r="E118" s="26" t="n"/>
+      <c r="F118" s="14" t="inlineStr">
+        <is>
+          <t>Compétence</t>
+        </is>
+      </c>
+      <c r="G118" s="14" t="inlineStr">
+        <is>
+          <t>Carac</t>
+        </is>
+      </c>
+      <c r="H118" s="14" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+      <c r="I118" s="14" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="J118" s="26" t="n"/>
+      <c r="K118" s="20" t="inlineStr">
         <is>
           <t>Proprioception</t>
         </is>
       </c>
-      <c r="L118" s="11" t="n">
-        <v>10</v>
+      <c r="L118" s="21" t="inlineStr">
+        <is>
+          <t>INS</t>
+        </is>
       </c>
       <c r="M118" s="11" t="n">
         <v>0</v>
       </c>
       <c r="N118" s="12">
-        <f>(10-L118)*-20</f>
+        <f>M118+H24</f>
         <v/>
       </c>
     </row>
     <row r="119">
-      <c r="F119" s="14" t="inlineStr">
+      <c r="A119" s="26" t="n"/>
+      <c r="B119" s="26" t="n"/>
+      <c r="C119" s="26" t="n"/>
+      <c r="D119" s="26" t="n"/>
+      <c r="E119" s="26" t="n"/>
+      <c r="F119" s="20" t="inlineStr">
+        <is>
+          <t>Peinture &amp; dessin</t>
+        </is>
+      </c>
+      <c r="G119" s="21" t="inlineStr">
+        <is>
+          <t>IMA</t>
+        </is>
+      </c>
+      <c r="H119" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I119" s="12">
+        <f>H119+H26</f>
+        <v/>
+      </c>
+      <c r="J119" s="26" t="n"/>
+      <c r="K119" s="20" t="inlineStr">
+        <is>
+          <t>Thermoception</t>
+        </is>
+      </c>
+      <c r="L119" s="21" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="M119" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N119" s="12">
+        <f>M119+C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="19" t="inlineStr">
+        <is>
+          <t>Champ Transport</t>
+        </is>
+      </c>
+      <c r="B120" s="9" t="n"/>
+      <c r="C120" s="9" t="n"/>
+      <c r="D120" s="10" t="n"/>
+      <c r="E120" s="26" t="n"/>
+      <c r="F120" s="20" t="inlineStr">
+        <is>
+          <t>Écriture</t>
+        </is>
+      </c>
+      <c r="G120" s="21" t="inlineStr">
+        <is>
+          <t>IMA</t>
+        </is>
+      </c>
+      <c r="H120" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I120" s="12">
+        <f>H120+H26</f>
+        <v/>
+      </c>
+      <c r="J120" s="26" t="n"/>
+      <c r="K120" s="20" t="inlineStr">
+        <is>
+          <t>Séismoréception</t>
+        </is>
+      </c>
+      <c r="L120" s="21" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="M120" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N120" s="12">
+        <f>M120+C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="14" t="inlineStr">
         <is>
           <t>Compétence</t>
         </is>
       </c>
-      <c r="G119" s="14" t="inlineStr">
+      <c r="B121" s="14" t="inlineStr">
         <is>
           <t>Carac</t>
         </is>
       </c>
-      <c r="H119" s="14" t="inlineStr">
+      <c r="C121" s="14" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="I119" s="14" t="inlineStr">
+      <c r="D121" s="14" t="inlineStr">
         <is>
           <t>Bonus</t>
         </is>
       </c>
-      <c r="K119" s="20" t="inlineStr">
-        <is>
-          <t>Thermoception</t>
-        </is>
-      </c>
-      <c r="L119" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="M119" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N119" s="12">
-        <f>(10-L119)*-20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="120">
-      <c r="F120" s="20" t="inlineStr">
-        <is>
-          <t>Forge / Métallurgie</t>
-        </is>
-      </c>
-      <c r="G120" s="21" t="inlineStr">
+      <c r="E121" s="26" t="n"/>
+      <c r="F121" s="20" t="inlineStr">
+        <is>
+          <t>Conte / Narration</t>
+        </is>
+      </c>
+      <c r="G121" s="21" t="inlineStr">
+        <is>
+          <t>CHA</t>
+        </is>
+      </c>
+      <c r="H121" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" s="12">
+        <f>H121+H27</f>
+        <v/>
+      </c>
+      <c r="J121" s="26" t="n"/>
+      <c r="K121" s="26" t="n"/>
+      <c r="L121" s="26" t="n"/>
+      <c r="M121" s="26" t="n"/>
+      <c r="N121" s="26" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="20" t="inlineStr">
+        <is>
+          <t>Conduite</t>
+        </is>
+      </c>
+      <c r="B122" s="21" t="inlineStr">
         <is>
           <t>DEX</t>
         </is>
       </c>
-      <c r="H120" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I120" s="12">
-        <f>H120+C23</f>
-        <v/>
-      </c>
-      <c r="K120" s="13" t="inlineStr">
-        <is>
-          <t>Malus perception = (10−acuité)×−20 (affiché). Malus d'action = (10−acuité)×−10.</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="F121" s="22" t="inlineStr">
-        <is>
-          <t>Travail du bois</t>
-        </is>
-      </c>
-      <c r="G121" s="23" t="inlineStr">
+      <c r="C122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D122" s="12">
+        <f>C122+C23</f>
+        <v/>
+      </c>
+      <c r="E122" s="26" t="n"/>
+      <c r="F122" s="20" t="inlineStr">
+        <is>
+          <t>Musique</t>
+        </is>
+      </c>
+      <c r="G122" s="21" t="inlineStr">
+        <is>
+          <t>IMA</t>
+        </is>
+      </c>
+      <c r="H122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" s="12">
+        <f>H122+H26</f>
+        <v/>
+      </c>
+      <c r="J122" s="26" t="n"/>
+      <c r="K122" s="19" t="inlineStr">
+        <is>
+          <t>Champ Technique</t>
+        </is>
+      </c>
+      <c r="L122" s="9" t="n"/>
+      <c r="M122" s="9" t="n"/>
+      <c r="N122" s="10" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="20" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B123" s="21" t="inlineStr">
         <is>
           <t>DEX</t>
         </is>
       </c>
-      <c r="H121" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I121" s="12">
-        <f>H121+C23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="122">
-      <c r="F122" s="20" t="inlineStr">
-        <is>
-          <t>Travail de la pierre</t>
-        </is>
-      </c>
-      <c r="G122" s="21" t="inlineStr">
+      <c r="C123" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" s="12">
+        <f>C123+C23</f>
+        <v/>
+      </c>
+      <c r="E123" s="26" t="n"/>
+      <c r="F123" s="20" t="inlineStr">
+        <is>
+          <t>Chant</t>
+        </is>
+      </c>
+      <c r="G123" s="21" t="inlineStr">
+        <is>
+          <t>CHA</t>
+        </is>
+      </c>
+      <c r="H123" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I123" s="12">
+        <f>H123+H27</f>
+        <v/>
+      </c>
+      <c r="J123" s="26" t="n"/>
+      <c r="K123" s="14" t="inlineStr">
+        <is>
+          <t>Compétence</t>
+        </is>
+      </c>
+      <c r="L123" s="14" t="inlineStr">
+        <is>
+          <t>Carac</t>
+        </is>
+      </c>
+      <c r="M123" s="14" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+      <c r="N123" s="14" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="20" t="inlineStr">
+        <is>
+          <t>Pilotage</t>
+        </is>
+      </c>
+      <c r="B124" s="21" t="inlineStr">
         <is>
           <t>DEX</t>
         </is>
       </c>
-      <c r="H122" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I122" s="12">
-        <f>H122+C23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="123">
-      <c r="F123" s="22" t="inlineStr">
-        <is>
-          <t>Textile</t>
-        </is>
-      </c>
-      <c r="G123" s="23" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
-      <c r="H123" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I123" s="12">
-        <f>H123+C23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="124">
+      <c r="C124" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" s="12">
+        <f>C124+C23</f>
+        <v/>
+      </c>
+      <c r="E124" s="26" t="n"/>
       <c r="F124" s="20" t="inlineStr">
         <is>
-          <t>Travail du cuir</t>
+          <t>Danse</t>
         </is>
       </c>
       <c r="G124" s="21" t="inlineStr">
         <is>
-          <t>DEX</t>
+          <t>AGI</t>
         </is>
       </c>
       <c r="H124" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I124" s="12">
-        <f>H124+C23</f>
+        <f>H124+C24</f>
+        <v/>
+      </c>
+      <c r="J124" s="26" t="n"/>
+      <c r="K124" s="20" t="inlineStr">
+        <is>
+          <t>Mécanique</t>
+        </is>
+      </c>
+      <c r="L124" s="21" t="inlineStr">
+        <is>
+          <t>LOG</t>
+        </is>
+      </c>
+      <c r="M124" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" s="12">
+        <f>M124+H23</f>
         <v/>
       </c>
     </row>
     <row r="125">
-      <c r="F125" s="22" t="inlineStr">
-        <is>
-          <t>Poterie &amp; verre</t>
-        </is>
-      </c>
-      <c r="G125" s="23" t="inlineStr">
-        <is>
-          <t>DEX</t>
+      <c r="A125" s="20" t="inlineStr">
+        <is>
+          <t>Équitation</t>
+        </is>
+      </c>
+      <c r="B125" s="21" t="inlineStr">
+        <is>
+          <t>AGI</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" s="12">
+        <f>C125+C24</f>
+        <v/>
+      </c>
+      <c r="E125" s="26" t="n"/>
+      <c r="F125" s="20" t="inlineStr">
+        <is>
+          <t>Personnification</t>
+        </is>
+      </c>
+      <c r="G125" s="21" t="inlineStr">
+        <is>
+          <t>CHA</t>
         </is>
       </c>
       <c r="H125" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I125" s="12">
-        <f>H125+C23</f>
+        <f>H125+H27</f>
+        <v/>
+      </c>
+      <c r="J125" s="26" t="n"/>
+      <c r="K125" s="20" t="inlineStr">
+        <is>
+          <t>Électronique</t>
+        </is>
+      </c>
+      <c r="L125" s="21" t="inlineStr">
+        <is>
+          <t>LOG</t>
+        </is>
+      </c>
+      <c r="M125" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N125" s="12">
+        <f>M125+H23</f>
         <v/>
       </c>
     </row>
     <row r="126">
-      <c r="F126" s="20" t="inlineStr">
-        <is>
-          <t>Joaillerie</t>
-        </is>
-      </c>
-      <c r="G126" s="21" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
-      <c r="H126" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I126" s="12">
-        <f>H126+C23</f>
+      <c r="A126" s="20" t="inlineStr">
+        <is>
+          <t>Glisse</t>
+        </is>
+      </c>
+      <c r="B126" s="21" t="inlineStr">
+        <is>
+          <t>AGI</t>
+        </is>
+      </c>
+      <c r="C126" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" s="12">
+        <f>C126+C24</f>
+        <v/>
+      </c>
+      <c r="E126" s="26" t="n"/>
+      <c r="F126" s="27" t="n"/>
+      <c r="G126" s="28" t="n"/>
+      <c r="H126" s="28" t="n"/>
+      <c r="I126" s="28" t="n"/>
+      <c r="J126" s="26" t="n"/>
+      <c r="K126" s="20" t="inlineStr">
+        <is>
+          <t>Programmation</t>
+        </is>
+      </c>
+      <c r="L126" s="21" t="inlineStr">
+        <is>
+          <t>LOG</t>
+        </is>
+      </c>
+      <c r="M126" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" s="12">
+        <f>M126+H23</f>
         <v/>
       </c>
     </row>
     <row r="127">
-      <c r="F127" s="22" t="inlineStr">
-        <is>
-          <t>Cuisine</t>
-        </is>
-      </c>
-      <c r="G127" s="23" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
-      <c r="H127" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I127" s="12">
-        <f>H127+C23</f>
+      <c r="A127" s="26" t="n"/>
+      <c r="B127" s="26" t="n"/>
+      <c r="C127" s="26" t="n"/>
+      <c r="D127" s="26" t="n"/>
+      <c r="E127" s="26" t="n"/>
+      <c r="F127" s="27" t="n"/>
+      <c r="G127" s="28" t="n"/>
+      <c r="H127" s="28" t="n"/>
+      <c r="I127" s="28" t="n"/>
+      <c r="J127" s="26" t="n"/>
+      <c r="K127" s="20" t="inlineStr">
+        <is>
+          <t>Cybersécurité</t>
+        </is>
+      </c>
+      <c r="L127" s="21" t="inlineStr">
+        <is>
+          <t>LOG</t>
+        </is>
+      </c>
+      <c r="M127" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" s="12">
+        <f>M127+H23</f>
         <v/>
       </c>
     </row>
     <row r="128">
-      <c r="F128" s="20" t="inlineStr">
-        <is>
-          <t>Brasserie &amp; distillation</t>
-        </is>
-      </c>
-      <c r="G128" s="21" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
-      <c r="H128" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I128" s="12">
-        <f>H128+C23</f>
+      <c r="A128" s="26" t="n"/>
+      <c r="B128" s="26" t="n"/>
+      <c r="C128" s="26" t="n"/>
+      <c r="D128" s="26" t="n"/>
+      <c r="E128" s="26" t="n"/>
+      <c r="F128" s="27" t="n"/>
+      <c r="G128" s="28" t="n"/>
+      <c r="H128" s="28" t="n"/>
+      <c r="I128" s="28" t="n"/>
+      <c r="J128" s="26" t="n"/>
+      <c r="K128" s="20" t="inlineStr">
+        <is>
+          <t>Réseaux &amp; télécoms</t>
+        </is>
+      </c>
+      <c r="L128" s="21" t="inlineStr">
+        <is>
+          <t>LOG</t>
+        </is>
+      </c>
+      <c r="M128" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" s="12">
+        <f>M128+H23</f>
         <v/>
       </c>
     </row>
     <row r="129">
-      <c r="F129" s="22" t="inlineStr">
-        <is>
-          <t>Parfumerie</t>
-        </is>
-      </c>
-      <c r="G129" s="23" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
-      <c r="H129" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I129" s="12">
-        <f>H129+C23</f>
+      <c r="A129" s="26" t="n"/>
+      <c r="B129" s="26" t="n"/>
+      <c r="C129" s="26" t="n"/>
+      <c r="D129" s="26" t="n"/>
+      <c r="E129" s="26" t="n"/>
+      <c r="F129" s="27" t="n"/>
+      <c r="G129" s="28" t="n"/>
+      <c r="H129" s="28" t="n"/>
+      <c r="I129" s="28" t="n"/>
+      <c r="J129" s="26" t="n"/>
+      <c r="K129" s="20" t="inlineStr">
+        <is>
+          <t>Cryptographie</t>
+        </is>
+      </c>
+      <c r="L129" s="21" t="inlineStr">
+        <is>
+          <t>LOG</t>
+        </is>
+      </c>
+      <c r="M129" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N129" s="12">
+        <f>M129+H23</f>
         <v/>
       </c>
     </row>
     <row r="130">
-      <c r="F130" s="20" t="inlineStr">
-        <is>
-          <t>Calligraphie</t>
-        </is>
-      </c>
-      <c r="G130" s="21" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
-      <c r="H130" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I130" s="12">
-        <f>H130+C23</f>
+      <c r="A130" s="26" t="n"/>
+      <c r="B130" s="26" t="n"/>
+      <c r="C130" s="26" t="n"/>
+      <c r="D130" s="26" t="n"/>
+      <c r="E130" s="26" t="n"/>
+      <c r="F130" s="27" t="n"/>
+      <c r="G130" s="28" t="n"/>
+      <c r="H130" s="28" t="n"/>
+      <c r="I130" s="28" t="n"/>
+      <c r="J130" s="26" t="n"/>
+      <c r="K130" s="20" t="inlineStr">
+        <is>
+          <t>Chimie</t>
+        </is>
+      </c>
+      <c r="L130" s="21" t="inlineStr">
+        <is>
+          <t>ÉRU</t>
+        </is>
+      </c>
+      <c r="M130" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N130" s="12">
+        <f>M130+H25</f>
         <v/>
       </c>
     </row>
     <row r="131">
-      <c r="F131" s="22" t="inlineStr">
-        <is>
-          <t>Peinture &amp; dessin</t>
-        </is>
-      </c>
-      <c r="G131" s="23" t="inlineStr">
-        <is>
-          <t>IMA</t>
-        </is>
-      </c>
-      <c r="H131" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I131" s="12">
-        <f>H131+H26</f>
+      <c r="A131" s="26" t="n"/>
+      <c r="B131" s="26" t="n"/>
+      <c r="C131" s="26" t="n"/>
+      <c r="D131" s="26" t="n"/>
+      <c r="E131" s="26" t="n"/>
+      <c r="F131" s="27" t="n"/>
+      <c r="G131" s="28" t="n"/>
+      <c r="H131" s="28" t="n"/>
+      <c r="I131" s="28" t="n"/>
+      <c r="J131" s="26" t="n"/>
+      <c r="K131" s="20" t="inlineStr">
+        <is>
+          <t>Pharmacologie</t>
+        </is>
+      </c>
+      <c r="L131" s="21" t="inlineStr">
+        <is>
+          <t>ÉRU</t>
+        </is>
+      </c>
+      <c r="M131" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N131" s="12">
+        <f>M131+H25</f>
         <v/>
       </c>
     </row>
     <row r="132">
-      <c r="F132" s="20" t="inlineStr">
-        <is>
-          <t>Écriture</t>
-        </is>
-      </c>
-      <c r="G132" s="21" t="inlineStr">
-        <is>
-          <t>IMA</t>
-        </is>
-      </c>
-      <c r="H132" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I132" s="12">
-        <f>H132+H26</f>
+      <c r="A132" s="26" t="n"/>
+      <c r="B132" s="26" t="n"/>
+      <c r="C132" s="26" t="n"/>
+      <c r="D132" s="26" t="n"/>
+      <c r="E132" s="26" t="n"/>
+      <c r="F132" s="27" t="n"/>
+      <c r="G132" s="28" t="n"/>
+      <c r="H132" s="28" t="n"/>
+      <c r="I132" s="28" t="n"/>
+      <c r="J132" s="26" t="n"/>
+      <c r="K132" s="20" t="inlineStr">
+        <is>
+          <t>Explosifs</t>
+        </is>
+      </c>
+      <c r="L132" s="21" t="inlineStr">
+        <is>
+          <t>ÉRU</t>
+        </is>
+      </c>
+      <c r="M132" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N132" s="12">
+        <f>M132+H25</f>
         <v/>
       </c>
     </row>
     <row r="133">
-      <c r="F133" s="22" t="inlineStr">
-        <is>
-          <t>Conte / Narration</t>
-        </is>
-      </c>
-      <c r="G133" s="23" t="inlineStr">
-        <is>
-          <t>CHA</t>
-        </is>
-      </c>
-      <c r="H133" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I133" s="12">
-        <f>H133+H27</f>
-        <v/>
-      </c>
+      <c r="A133" s="26" t="n"/>
+      <c r="B133" s="26" t="n"/>
+      <c r="C133" s="26" t="n"/>
+      <c r="D133" s="26" t="n"/>
+      <c r="E133" s="26" t="n"/>
+      <c r="F133" s="27" t="n"/>
+      <c r="G133" s="28" t="n"/>
+      <c r="H133" s="28" t="n"/>
+      <c r="I133" s="28" t="n"/>
+      <c r="J133" s="26" t="n"/>
+      <c r="K133" s="26" t="n"/>
+      <c r="L133" s="26" t="n"/>
+      <c r="M133" s="26" t="n"/>
+      <c r="N133" s="26" t="n"/>
     </row>
     <row r="134">
-      <c r="F134" s="20" t="inlineStr">
-        <is>
-          <t>Musique &amp; chant</t>
-        </is>
-      </c>
-      <c r="G134" s="21" t="inlineStr">
-        <is>
-          <t>IMA</t>
-        </is>
-      </c>
-      <c r="H134" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I134" s="12">
-        <f>H134+H26</f>
-        <v/>
-      </c>
+      <c r="A134" s="26" t="n"/>
+      <c r="B134" s="26" t="n"/>
+      <c r="C134" s="26" t="n"/>
+      <c r="D134" s="26" t="n"/>
+      <c r="E134" s="26" t="n"/>
+      <c r="F134" s="27" t="n"/>
+      <c r="G134" s="28" t="n"/>
+      <c r="H134" s="28" t="n"/>
+      <c r="I134" s="28" t="n"/>
+      <c r="J134" s="26" t="n"/>
+      <c r="K134" s="26" t="n"/>
+      <c r="L134" s="26" t="n"/>
+      <c r="M134" s="26" t="n"/>
+      <c r="N134" s="26" t="n"/>
     </row>
     <row r="135">
-      <c r="F135" s="22" t="inlineStr">
-        <is>
-          <t>Danse</t>
-        </is>
-      </c>
-      <c r="G135" s="23" t="inlineStr">
-        <is>
-          <t>AGI</t>
-        </is>
-      </c>
-      <c r="H135" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I135" s="12">
-        <f>H135+C24</f>
-        <v/>
-      </c>
+      <c r="A135" s="26" t="n"/>
+      <c r="B135" s="26" t="n"/>
+      <c r="C135" s="26" t="n"/>
+      <c r="D135" s="26" t="n"/>
+      <c r="E135" s="26" t="n"/>
+      <c r="F135" s="27" t="n"/>
+      <c r="G135" s="28" t="n"/>
+      <c r="H135" s="28" t="n"/>
+      <c r="I135" s="28" t="n"/>
+      <c r="J135" s="26" t="n"/>
+      <c r="K135" s="26" t="n"/>
+      <c r="L135" s="26" t="n"/>
+      <c r="M135" s="26" t="n"/>
+      <c r="N135" s="26" t="n"/>
     </row>
     <row r="136">
-      <c r="F136" s="20" t="inlineStr">
-        <is>
-          <t>Théâtre</t>
-        </is>
-      </c>
-      <c r="G136" s="21" t="inlineStr">
-        <is>
-          <t>CHA</t>
-        </is>
-      </c>
-      <c r="H136" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I136" s="12">
-        <f>H136+H27</f>
-        <v/>
-      </c>
+      <c r="A136" s="26" t="n"/>
+      <c r="B136" s="26" t="n"/>
+      <c r="C136" s="26" t="n"/>
+      <c r="D136" s="26" t="n"/>
+      <c r="E136" s="26" t="n"/>
+      <c r="F136" s="27" t="n"/>
+      <c r="G136" s="28" t="n"/>
+      <c r="H136" s="28" t="n"/>
+      <c r="I136" s="28" t="n"/>
+      <c r="J136" s="26" t="n"/>
+      <c r="K136" s="26" t="n"/>
+      <c r="L136" s="26" t="n"/>
+      <c r="M136" s="26" t="n"/>
+      <c r="N136" s="26" t="n"/>
     </row>
     <row r="137">
-      <c r="F137" s="22" t="inlineStr">
-        <is>
-          <t>Marionnettes</t>
-        </is>
-      </c>
-      <c r="G137" s="23" t="inlineStr">
-        <is>
-          <t>DEX</t>
-        </is>
-      </c>
-      <c r="H137" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I137" s="12">
-        <f>H137+C23</f>
-        <v/>
-      </c>
+      <c r="A137" s="26" t="n"/>
+      <c r="B137" s="26" t="n"/>
+      <c r="C137" s="26" t="n"/>
+      <c r="D137" s="26" t="n"/>
+      <c r="E137" s="26" t="n"/>
+      <c r="F137" s="27" t="n"/>
+      <c r="G137" s="28" t="n"/>
+      <c r="H137" s="28" t="n"/>
+      <c r="I137" s="28" t="n"/>
+      <c r="J137" s="26" t="n"/>
+      <c r="K137" s="26" t="n"/>
+      <c r="L137" s="26" t="n"/>
+      <c r="M137" s="26" t="n"/>
+      <c r="N137" s="26" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="26" t="n"/>
+      <c r="B138" s="26" t="n"/>
+      <c r="C138" s="26" t="n"/>
+      <c r="D138" s="26" t="n"/>
+      <c r="E138" s="26" t="n"/>
+      <c r="F138" s="26" t="n"/>
+      <c r="G138" s="26" t="n"/>
+      <c r="H138" s="26" t="n"/>
+      <c r="I138" s="26" t="n"/>
+      <c r="J138" s="26" t="n"/>
+      <c r="K138" s="26" t="n"/>
+      <c r="L138" s="26" t="n"/>
+      <c r="M138" s="26" t="n"/>
+      <c r="N138" s="26" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="26" t="n"/>
+      <c r="B139" s="26" t="n"/>
+      <c r="C139" s="26" t="n"/>
+      <c r="D139" s="26" t="n"/>
+      <c r="E139" s="26" t="n"/>
+      <c r="F139" s="26" t="n"/>
+      <c r="G139" s="26" t="n"/>
+      <c r="H139" s="26" t="n"/>
+      <c r="I139" s="26" t="n"/>
+      <c r="J139" s="26" t="n"/>
+      <c r="K139" s="26" t="n"/>
+      <c r="L139" s="26" t="n"/>
+      <c r="M139" s="26" t="n"/>
+      <c r="N139" s="26" t="n"/>
     </row>
     <row r="140" ht="26" customHeight="1">
       <c r="A140" s="24" t="inlineStr">
@@ -4802,7 +5407,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="44">
     <mergeCell ref="H35:I35"/>
     <mergeCell ref="F56:I56"/>
     <mergeCell ref="F102:I102"/>
@@ -4811,9 +5416,11 @@
     <mergeCell ref="A100:D100"/>
     <mergeCell ref="E31:G31"/>
     <mergeCell ref="A64:N64"/>
+    <mergeCell ref="A109:D109"/>
     <mergeCell ref="F77:I77"/>
     <mergeCell ref="F92:I92"/>
     <mergeCell ref="G34:I34"/>
+    <mergeCell ref="F117:I117"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="C28:I28"/>
@@ -4824,27 +5431,27 @@
     <mergeCell ref="A46:N46"/>
     <mergeCell ref="A18:N18"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="F118:I118"/>
     <mergeCell ref="A10:N10"/>
     <mergeCell ref="A12:N12"/>
+    <mergeCell ref="K21:N21"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A87:D87"/>
     <mergeCell ref="G9:I9"/>
     <mergeCell ref="A76:N76"/>
+    <mergeCell ref="K122:N122"/>
     <mergeCell ref="A58:I58"/>
     <mergeCell ref="A42:N42"/>
     <mergeCell ref="B49:C49"/>
-    <mergeCell ref="A108:D108"/>
     <mergeCell ref="B74:C74"/>
+    <mergeCell ref="K106:N106"/>
     <mergeCell ref="A140:N140"/>
+    <mergeCell ref="A120:D120"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="A20:N20"/>
-    <mergeCell ref="K105:N105"/>
     <mergeCell ref="K77:N77"/>
     <mergeCell ref="F74:N74"/>
     <mergeCell ref="I31:J31"/>
     <mergeCell ref="A40:A41"/>
-    <mergeCell ref="K120:N120"/>
   </mergeCells>
   <dataValidations count="20">
     <dataValidation sqref="G5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4944,7 +5551,7 @@
           <t>MOD carac (valeur 0–30 → modificateur)</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n"/>
+      <c r="B3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
@@ -5212,7 +5819,7 @@
           <t>Plafond carac par Éclat</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n"/>
+      <c r="B37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
@@ -5280,9 +5887,9 @@
           <t>Création par Éclat (moyenne / plafond / budget)</t>
         </is>
       </c>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="6" t="n"/>
-      <c r="D46" s="6" t="n"/>
+      <c r="B46" s="9" t="n"/>
+      <c r="C46" s="9" t="n"/>
+      <c r="D46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
@@ -5368,9 +5975,9 @@
           <t>Indice de poids (FOR → Légère / Inter / Lourde)</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-      <c r="D53" s="6" t="n"/>
+      <c r="B53" s="9" t="n"/>
+      <c r="C53" s="9" t="n"/>
+      <c r="D53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
@@ -5400,17 +6007,17 @@
       </c>
       <c r="B55" s="23" t="inlineStr">
         <is>
-          <t>&lt;1 kg</t>
+          <t>0 kg</t>
         </is>
       </c>
       <c r="C55" s="23" t="inlineStr">
         <is>
-          <t>1 kg</t>
+          <t>0 kg</t>
         </is>
       </c>
       <c r="D55" s="23" t="inlineStr">
         <is>
-          <t>2 kg</t>
+          <t>0 kg</t>
         </is>
       </c>
     </row>
@@ -6020,9 +6627,9 @@
           <t>Mouvement (AGI → Légère / Inter / Lourde, par round)</t>
         </is>
       </c>
-      <c r="B87" s="6" t="n"/>
-      <c r="C87" s="6" t="n"/>
-      <c r="D87" s="6" t="n"/>
+      <c r="B87" s="9" t="n"/>
+      <c r="C87" s="9" t="n"/>
+      <c r="D87" s="10" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
@@ -6052,17 +6659,17 @@
       </c>
       <c r="B89" s="23" t="inlineStr">
         <is>
-          <t>1 m</t>
+          <t>0 m</t>
         </is>
       </c>
       <c r="C89" s="23" t="inlineStr">
         <is>
-          <t>2 m</t>
+          <t>0 m</t>
         </is>
       </c>
       <c r="D89" s="23" t="inlineStr">
         <is>
-          <t>5 m</t>
+          <t>0 m</t>
         </is>
       </c>
     </row>
@@ -6672,9 +7279,9 @@
           <t>Apnée (END → Légère / Inter / Lourde)</t>
         </is>
       </c>
-      <c r="B121" s="6" t="n"/>
-      <c r="C121" s="6" t="n"/>
-      <c r="D121" s="6" t="n"/>
+      <c r="B121" s="9" t="n"/>
+      <c r="C121" s="9" t="n"/>
+      <c r="D121" s="10" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
@@ -7324,13 +7931,13 @@
           <t>Affinités par archétype (%)  —  G = Spé sans Spécialiste, H = Spé avec</t>
         </is>
       </c>
-      <c r="B155" s="6" t="n"/>
-      <c r="C155" s="6" t="n"/>
-      <c r="D155" s="6" t="n"/>
-      <c r="E155" s="6" t="n"/>
-      <c r="F155" s="6" t="n"/>
-      <c r="G155" s="6" t="n"/>
-      <c r="H155" s="6" t="n"/>
+      <c r="B155" s="9" t="n"/>
+      <c r="C155" s="9" t="n"/>
+      <c r="D155" s="9" t="n"/>
+      <c r="E155" s="9" t="n"/>
+      <c r="F155" s="9" t="n"/>
+      <c r="G155" s="9" t="n"/>
+      <c r="H155" s="10" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="14" t="inlineStr">
@@ -7716,11 +8323,11 @@
           <t>Coûts DI des techniques (cumulés par palier)</t>
         </is>
       </c>
-      <c r="B170" s="6" t="n"/>
-      <c r="C170" s="6" t="n"/>
-      <c r="D170" s="6" t="n"/>
-      <c r="E170" s="6" t="n"/>
-      <c r="F170" s="6" t="n"/>
+      <c r="B170" s="9" t="n"/>
+      <c r="C170" s="9" t="n"/>
+      <c r="D170" s="9" t="n"/>
+      <c r="E170" s="9" t="n"/>
+      <c r="F170" s="10" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="14" t="inlineStr">
@@ -7914,7 +8521,7 @@
           <t>Base d'UAR par palier (état à manteau actif)</t>
         </is>
       </c>
-      <c r="B180" s="6" t="n"/>
+      <c r="B180" s="10" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="14" t="inlineStr">
@@ -7984,7 +8591,7 @@
           <t>Échelle de difficulté (palier → seuil)</t>
         </is>
       </c>
-      <c r="B188" s="6" t="n"/>
+      <c r="B188" s="10" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="14" t="inlineStr">
@@ -8134,9 +8741,9 @@
           <t>Types de dégâts (7)</t>
         </is>
       </c>
-      <c r="B204" s="6" t="n"/>
-      <c r="C204" s="6" t="n"/>
-      <c r="D204" s="6" t="n"/>
+      <c r="B204" s="9" t="n"/>
+      <c r="C204" s="9" t="n"/>
+      <c r="D204" s="10" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="14" t="inlineStr">
@@ -8320,8 +8927,8 @@
           <t>Rayon d'En (rayon → coût DI cumulé + aura/tour)</t>
         </is>
       </c>
-      <c r="B214" s="6" t="n"/>
-      <c r="C214" s="6" t="n"/>
+      <c r="B214" s="9" t="n"/>
+      <c r="C214" s="10" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="14" t="inlineStr">
@@ -8567,13 +9174,13 @@
           <t>RÉFÉRENCE — aide-mémoire (consultatif)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="9" t="n"/>
+      <c r="D1" s="9" t="n"/>
+      <c r="E1" s="9" t="n"/>
+      <c r="F1" s="9" t="n"/>
+      <c r="G1" s="9" t="n"/>
+      <c r="H1" s="10" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -8581,7 +9188,7 @@
           <t>Échelle de difficulté</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n"/>
+      <c r="B3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
@@ -8731,9 +9338,9 @@
           <t>Types de dégâts (7)</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
@@ -8917,7 +9524,7 @@
           <t>Marge (% de touche)</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n"/>
+      <c r="B29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
@@ -8985,8 +9592,8 @@
           <t>Postures de combat</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="6" t="n"/>
+      <c r="B36" s="9" t="n"/>
+      <c r="C36" s="10" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
@@ -9079,11 +9686,11 @@
           <t>Situations</t>
         </is>
       </c>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="6" t="n"/>
-      <c r="D43" s="6" t="n"/>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="6" t="n"/>
+      <c r="B43" s="9" t="n"/>
+      <c r="C43" s="9" t="n"/>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="9" t="n"/>
+      <c r="F43" s="10" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
@@ -9248,19 +9855,19 @@
     <row r="49">
       <c r="A49" s="22" t="inlineStr">
         <is>
-          <t>Position supérieure</t>
+          <t>Surpris</t>
         </is>
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
+          <t>−120</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
           <t>–</t>
         </is>
       </c>
-      <c r="C49" s="23" t="inlineStr">
-        <is>
-          <t>+20</t>
-        </is>
-      </c>
       <c r="D49" s="23" t="inlineStr">
         <is>
           <t>–</t>
@@ -9278,68 +9885,20 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="20" t="inlineStr">
-        <is>
-          <t>Position inférieure</t>
-        </is>
-      </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>−20</t>
-        </is>
-      </c>
-      <c r="D50" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E50" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F50" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
+      <c r="A50" s="29" t="n"/>
+      <c r="B50" s="30" t="n"/>
+      <c r="C50" s="30" t="n"/>
+      <c r="D50" s="30" t="n"/>
+      <c r="E50" s="30" t="n"/>
+      <c r="F50" s="30" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="22" t="inlineStr">
-        <is>
-          <t>Surpris</t>
-        </is>
-      </c>
-      <c r="B51" s="23" t="inlineStr">
-        <is>
-          <t>−120</t>
-        </is>
-      </c>
-      <c r="C51" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D51" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E51" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F51" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
+      <c r="A51" s="29" t="n"/>
+      <c r="B51" s="30" t="n"/>
+      <c r="C51" s="30" t="n"/>
+      <c r="D51" s="30" t="n"/>
+      <c r="E51" s="30" t="n"/>
+      <c r="F51" s="30" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
@@ -9347,7 +9906,7 @@
           <t>États / afflictions (malus)</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n"/>
+      <c r="B53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
@@ -9364,46 +9923,46 @@
     <row r="55">
       <c r="A55" s="22" t="inlineStr">
         <is>
+          <t>Prise</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="inlineStr">
+        <is>
+          <t>Agrippé / Maîtrisé / Soumis : saisi, mouvement 0 ; + Paralysie légère / partielle / totale</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="22" t="inlineStr">
+        <is>
           <t>Immobilisé</t>
         </is>
       </c>
-      <c r="B55" s="23" t="inlineStr">
-        <is>
-          <t>−20 att/esq ; +20 contre lui</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="20" t="inlineStr">
-        <is>
-          <t>Étourdi</t>
-        </is>
-      </c>
-      <c r="B56" s="21" t="inlineStr">
-        <is>
-          <t>perd actions, pas de réaction ; +20 contre lui</t>
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>entravé, mouvement 0 ; + Paralysie selon le degré</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="22" t="inlineStr">
         <is>
-          <t>À terre</t>
+          <t>Mutisme</t>
         </is>
       </c>
       <c r="B57" s="23" t="inlineStr">
         <is>
-          <t>−20 att ; +20 mêlée contre / −20 distance contre</t>
+          <t>Léger : −80 compétences Vocales · Partiel : muet (sons ok) · Total : aucun son</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="20" t="inlineStr">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>Paralysie légère</t>
         </is>
       </c>
-      <c r="B58" s="21" t="inlineStr">
+      <c r="B58" s="23" t="inlineStr">
         <is>
           <t>−20 att/par/init ; −40 esq/phys</t>
         </is>
@@ -9422,12 +9981,12 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="20" t="inlineStr">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>Paralysie totale</t>
         </is>
       </c>
-      <c r="B60" s="21" t="inlineStr">
+      <c r="B60" s="23" t="inlineStr">
         <is>
           <t>−200 att/par/esq/phys ; −100 init</t>
         </is>
@@ -9436,12 +9995,24 @@
     <row r="61">
       <c r="A61" s="22" t="inlineStr">
         <is>
+          <t>À terre</t>
+        </is>
+      </c>
+      <c r="B61" s="23" t="inlineStr">
+        <is>
+          <t>−20 att ; contre lui +20 mêlée / −20 distance ; relever = 1 action</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr">
+        <is>
           <t>Inconscience</t>
         </is>
       </c>
-      <c r="B61" s="23" t="inlineStr">
-        <is>
-          <t>toute attaque mêlée qui touche = critique</t>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>sans défense, touché automatiquement ; mêlée qui touche = critique ; tombe À terre</t>
         </is>
       </c>
     </row>
@@ -9451,7 +10022,7 @@
           <t>Manœuvres (malus à l'attaque)</t>
         </is>
       </c>
-      <c r="B63" s="6" t="n"/>
+      <c r="B63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
@@ -9543,7 +10114,7 @@
           <t>Viser (malus à l'attaque par zone)</t>
         </is>
       </c>
-      <c r="B72" s="6" t="n"/>
+      <c r="B72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
@@ -9659,10 +10230,10 @@
           <t>Catalogue d'armes (extrait — chaque arme vaut 100 points)</t>
         </is>
       </c>
-      <c r="B83" s="6" t="n"/>
-      <c r="C83" s="6" t="n"/>
-      <c r="D83" s="6" t="n"/>
-      <c r="E83" s="6" t="n"/>
+      <c r="B83" s="9" t="n"/>
+      <c r="C83" s="9" t="n"/>
+      <c r="D83" s="9" t="n"/>
+      <c r="E83" s="10" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="14" t="inlineStr">

</xml_diff>